<commit_message>
Update parameters except labour supply
</commit_message>
<xml_diff>
--- a/input/reg_fertility.xlsx
+++ b/input/reg_fertility.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FF51FC-7431-4262-8C45-7FA56BE9F970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D1F369-41F0-4695-94AC-40570846D454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="14566" windowHeight="17363" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
-    <sheet name="PL_F1a" sheetId="3" r:id="rId2"/>
-    <sheet name="PL_F1b" sheetId="4" r:id="rId3"/>
+    <sheet name="IT_F1a" sheetId="3" r:id="rId2"/>
+    <sheet name="IT_F1b" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="41">
   <si>
     <t>Description:</t>
   </si>
@@ -132,49 +132,36 @@
     <t>Y2020</t>
   </si>
   <si>
-    <t>PL4</t>
-  </si>
-  <si>
-    <t>PL5</t>
-  </si>
-  <si>
-    <t>PL6</t>
-  </si>
-  <si>
-    <t>Regions: PL4 = Polnocno-Zachodni, PL5 = Poludniowo-Zachodni, PL6 = Polnocy, PL10 = Central + East. Poludniowy is the omitted category.</t>
-  </si>
-  <si>
-    <t>PL10</t>
+    <t>Regions: ITF = South, ITG = Islands, ITH = Northeast, ITI = Central. Northwest (ITC) is the omitted region.</t>
+  </si>
+  <si>
+    <t>ITF</t>
+  </si>
+  <si>
+    <t>ITG</t>
+  </si>
+  <si>
+    <t>ITH</t>
+  </si>
+  <si>
+    <t>ITI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -187,28 +174,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -227,12 +193,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -568,7 +532,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
@@ -579,7 +543,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -603,11 +567,11 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -617,14 +581,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" t="s">
         <v>9</v>
       </c>
       <c r="C1" t="s">
@@ -637,126 +601,92 @@
         <v>12</v>
       </c>
       <c r="F1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4">
-        <v>-0.33877183111340164</v>
+      <c r="B2">
+        <v>-1.9658875381585693E-3</v>
       </c>
       <c r="C2">
-        <v>5.9273678788696743E-3</v>
+        <v>1.6312345539927151E-2</v>
       </c>
       <c r="D2">
-        <v>-8.0783036998965723E-4</v>
+        <v>-1.1828889899364998E-2</v>
       </c>
       <c r="E2">
-        <v>1.7426093405267219E-2</v>
+        <v>4.7442327799468692E-2</v>
       </c>
       <c r="F2">
-        <v>7.3003900325142018E-3</v>
-      </c>
-      <c r="G2">
-        <v>-0.13268969440411649</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A3" s="4" t="s">
+        <v>-0.35302933071638515</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="4">
-        <v>0.32659602149356004</v>
+      <c r="B3">
+        <v>0.14643989603547861</v>
       </c>
       <c r="C3">
-        <v>-8.0783036998965723E-4</v>
+        <v>-1.1828889899364998E-2</v>
       </c>
       <c r="D3">
-        <v>2.2626024511415942E-2</v>
+        <v>0.18750309379931057</v>
       </c>
       <c r="E3">
-        <v>5.10778215858438E-3</v>
+        <v>-0.15455786365213553</v>
       </c>
       <c r="F3">
-        <v>1.2537029016663603E-3</v>
-      </c>
-      <c r="G3">
-        <v>-8.0755321463503574E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A4" s="4" t="s">
+        <v>-0.42919776248276365</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="4">
-        <v>-0.96853811409855861</v>
+      <c r="B4">
+        <v>-0.48186314363830368</v>
       </c>
       <c r="C4">
-        <v>1.7426093405267219E-2</v>
+        <v>4.7442327799468692E-2</v>
       </c>
       <c r="D4">
-        <v>5.10778215858438E-3</v>
+        <v>-0.15455786365213553</v>
       </c>
       <c r="E4">
-        <v>0.14779296919533721</v>
+        <v>0.50907778618380339</v>
       </c>
       <c r="F4">
-        <v>9.0841112336903243E-2</v>
-      </c>
-      <c r="G4">
-        <v>-0.49105472984089227</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="4">
-        <v>-0.60092237408894833</v>
+        <v>-0.73373494833229547</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>-0.59270779555611164</v>
       </c>
       <c r="C5">
-        <v>7.3003900325142018E-3</v>
+        <v>-0.35302933071638515</v>
       </c>
       <c r="D5">
-        <v>1.2537029016663603E-3</v>
+        <v>-0.42919776248276365</v>
       </c>
       <c r="E5">
-        <v>9.0841112336903243E-2</v>
+        <v>-0.73373494833229547</v>
       </c>
       <c r="F5">
-        <v>0.34097859502626987</v>
-      </c>
-      <c r="G5">
-        <v>-0.24174421005554725</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="4">
-        <v>6.4673633509546748</v>
-      </c>
-      <c r="C6">
-        <v>-0.13268969440411649</v>
-      </c>
-      <c r="D6">
-        <v>-8.0755321463503574E-2</v>
-      </c>
-      <c r="E6">
-        <v>-0.49105472984089227</v>
-      </c>
-      <c r="F6">
-        <v>-0.24174421005554725</v>
-      </c>
-      <c r="G6">
-        <v>3.4723866729624069</v>
-      </c>
+        <v>10.430772870143954</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -772,10 +702,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A1" s="4" t="s">
+      <c r="A1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" t="s">
         <v>9</v>
       </c>
       <c r="C1" t="s">
@@ -842,13 +772,13 @@
         <v>33</v>
       </c>
       <c r="X1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Z1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AA1" t="s">
         <v>40</v>
@@ -867,2758 +797,2758 @@
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4">
-        <v>0.21222166754916791</v>
+      <c r="B2">
+        <v>0.25685035252636784</v>
       </c>
       <c r="C2">
-        <v>8.2670710700671977E-4</v>
+        <v>1.3521539366952381E-3</v>
       </c>
       <c r="D2">
-        <v>-1.1889967441694152E-5</v>
+        <v>-1.8754822350946112E-5</v>
       </c>
       <c r="E2">
-        <v>1.3954253592297309E-4</v>
+        <v>8.9056117468504226E-5</v>
       </c>
       <c r="F2">
-        <v>-1.5599553235947998E-4</v>
+        <v>6.7063061460856388E-5</v>
       </c>
       <c r="G2">
-        <v>-2.6702735423156908E-4</v>
+        <v>-9.5887305326766703E-5</v>
       </c>
       <c r="H2">
-        <v>-2.6739376720805869E-4</v>
+        <v>9.1379723694169634E-5</v>
       </c>
       <c r="I2">
-        <v>-3.3654092924715977E-4</v>
+        <v>-3.0072084295433218E-4</v>
       </c>
       <c r="J2">
-        <v>9.8342213252174994E-5</v>
+        <v>-9.0818006520796378E-5</v>
       </c>
       <c r="K2">
-        <v>-1.8877589968322069E-4</v>
+        <v>1.0206408574724157E-4</v>
       </c>
       <c r="L2">
-        <v>-1.0975709844830445E-4</v>
+        <v>1.1566475225018719E-4</v>
       </c>
       <c r="M2">
-        <v>-8.5185570430833853E-5</v>
+        <v>-4.0148122286011445E-5</v>
       </c>
       <c r="N2">
-        <v>-1.3499536097145645E-4</v>
+        <v>-8.9329145078764077E-5</v>
       </c>
       <c r="O2">
-        <v>7.6912382475424756E-5</v>
+        <v>-3.0777543329596566E-4</v>
       </c>
       <c r="P2">
-        <v>-1.1692880680639565E-4</v>
+        <v>1.7080749835791595E-5</v>
       </c>
       <c r="Q2">
-        <v>-7.3303706793806898E-5</v>
+        <v>1.520296086144089E-4</v>
       </c>
       <c r="R2">
-        <v>-2.5130572391913238E-4</v>
+        <v>-4.5032176654757634E-5</v>
       </c>
       <c r="S2">
-        <v>1.9243435626443449E-4</v>
+        <v>3.540702064387842E-5</v>
       </c>
       <c r="T2">
-        <v>4.4902128542772526E-4</v>
+        <v>1.5759634054272626E-4</v>
       </c>
       <c r="U2">
-        <v>2.3257402569426891E-4</v>
+        <v>6.7481258606760797E-4</v>
       </c>
       <c r="V2">
-        <v>1.036745703606724E-3</v>
+        <v>5.4872781593778841E-4</v>
       </c>
       <c r="W2">
-        <v>8.256034511573869E-5</v>
+        <v>1.3867767885126017E-4</v>
       </c>
       <c r="X2">
-        <v>4.255967225028686E-7</v>
+        <v>2.5913086894540846E-5</v>
       </c>
       <c r="Y2">
-        <v>-3.4369943042798063E-5</v>
+        <v>9.3965165858727467E-5</v>
       </c>
       <c r="Z2">
-        <v>5.7247109565838894E-6</v>
+        <v>-1.6917361960915034E-4</v>
       </c>
       <c r="AA2">
-        <v>-1.5838513064547559E-5</v>
+        <v>-3.875855575427925E-5</v>
       </c>
       <c r="AB2">
-        <v>5.9137605493958998E-6</v>
+        <v>2.7676159033733147E-5</v>
       </c>
       <c r="AC2">
-        <v>5.159375546955015E-5</v>
+        <v>-2.8837001124054889E-4</v>
       </c>
       <c r="AD2">
-        <v>2.5710270849494711E-5</v>
+        <v>-8.8906726277164852E-5</v>
       </c>
       <c r="AE2">
-        <v>-1.3815079267640334E-2</v>
+        <v>-2.4829431322037993E-2</v>
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A3" s="4" t="s">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="4">
-        <v>-4.4664697275741058E-3</v>
+      <c r="B3">
+        <v>-4.8096184442453487E-3</v>
       </c>
       <c r="C3">
-        <v>-1.1889967441694152E-5</v>
+        <v>-1.8754822350946112E-5</v>
       </c>
       <c r="D3">
-        <v>1.7303393143819542E-7</v>
+        <v>2.6308282537022193E-7</v>
       </c>
       <c r="E3">
-        <v>-2.1698517924429514E-6</v>
+        <v>-5.3490168679679387E-7</v>
       </c>
       <c r="F3">
-        <v>2.0828800479358259E-6</v>
+        <v>-1.2432081387031601E-7</v>
       </c>
       <c r="G3">
-        <v>3.6712026487779582E-6</v>
+        <v>1.4494476693503668E-6</v>
       </c>
       <c r="H3">
-        <v>3.4809970050741673E-6</v>
+        <v>-1.7199274866531414E-6</v>
       </c>
       <c r="I3">
-        <v>4.9164130985844696E-6</v>
+        <v>4.0778520476240335E-6</v>
       </c>
       <c r="J3">
-        <v>-8.4759990998648817E-7</v>
+        <v>2.1578858707211663E-6</v>
       </c>
       <c r="K3">
-        <v>3.0324858947823705E-6</v>
+        <v>-1.4554829651541759E-6</v>
       </c>
       <c r="L3">
-        <v>2.2771119802513846E-6</v>
+        <v>-1.5482169949105717E-6</v>
       </c>
       <c r="M3">
-        <v>2.0995616541072575E-6</v>
+        <v>9.6509726436080608E-7</v>
       </c>
       <c r="N3">
-        <v>3.0967256168015677E-6</v>
+        <v>1.4300579061547161E-6</v>
       </c>
       <c r="O3">
-        <v>-1.2798079003760058E-6</v>
+        <v>3.7347654422265314E-6</v>
       </c>
       <c r="P3">
-        <v>2.0231536991994901E-6</v>
+        <v>-4.9467523507792E-7</v>
       </c>
       <c r="Q3">
-        <v>1.7874509792603665E-6</v>
+        <v>-1.6566145337345119E-6</v>
       </c>
       <c r="R3">
-        <v>3.9857705274844041E-6</v>
+        <v>6.1326581762181589E-7</v>
       </c>
       <c r="S3">
-        <v>-2.8319923634328983E-6</v>
+        <v>-9.1955951857247437E-9</v>
       </c>
       <c r="T3">
-        <v>-6.4012366243920116E-6</v>
+        <v>-1.9322631231452825E-6</v>
       </c>
       <c r="U3">
-        <v>-2.9933107869743519E-6</v>
+        <v>-1.4569497607665009E-6</v>
       </c>
       <c r="V3">
-        <v>-1.417677093281909E-5</v>
+        <v>-7.0509937480622278E-6</v>
       </c>
       <c r="W3">
-        <v>-9.7725192968876098E-7</v>
+        <v>-2.2688969186693666E-6</v>
       </c>
       <c r="X3">
-        <v>-9.8252358527322638E-9</v>
+        <v>-7.9257668560221402E-7</v>
       </c>
       <c r="Y3">
-        <v>4.5168458805109964E-7</v>
+        <v>-1.4457021524091158E-6</v>
       </c>
       <c r="Z3">
-        <v>1.5333999195543346E-8</v>
+        <v>2.4065892310144482E-6</v>
       </c>
       <c r="AA3">
-        <v>2.6570736051742815E-7</v>
+        <v>3.0475044868048156E-7</v>
       </c>
       <c r="AB3">
-        <v>-1.1857098752095007E-7</v>
+        <v>-2.0298817239389688E-7</v>
       </c>
       <c r="AC3">
-        <v>-8.1506749543800876E-7</v>
+        <v>3.7089664899785427E-6</v>
       </c>
       <c r="AD3">
-        <v>-4.0582316391967095E-7</v>
+        <v>1.0264545465087224E-6</v>
       </c>
       <c r="AE3">
-        <v>1.9533488433813129E-4</v>
+        <v>3.2634569391603403E-4</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A4" s="4" t="s">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="4">
-        <v>0.31855061702804771</v>
+      <c r="B4">
+        <v>-0.29118186561899223</v>
       </c>
       <c r="C4">
-        <v>1.3954253592297309E-4</v>
+        <v>8.9056117468504226E-5</v>
       </c>
       <c r="D4">
-        <v>-2.1698517924429514E-6</v>
+        <v>-5.3490168679679387E-7</v>
       </c>
       <c r="E4">
-        <v>1.8517432113345257E-2</v>
+        <v>2.4237931065596883E-2</v>
       </c>
       <c r="F4">
-        <v>1.1320569731069548E-2</v>
+        <v>1.5644749416402162E-2</v>
       </c>
       <c r="G4">
-        <v>1.1280306269238073E-2</v>
+        <v>1.5527379691744369E-2</v>
       </c>
       <c r="H4">
-        <v>1.1290573524496765E-2</v>
+        <v>1.5418119334999938E-2</v>
       </c>
       <c r="I4">
-        <v>6.7062584488728307E-5</v>
+        <v>-1.0753962923125821E-3</v>
       </c>
       <c r="J4">
-        <v>1.9036617985941987E-5</v>
+        <v>1.0366554294107006E-3</v>
       </c>
       <c r="K4">
-        <v>2.8581898359109591E-4</v>
+        <v>-7.7187129409041037E-5</v>
       </c>
       <c r="L4">
-        <v>1.9187935253608566E-4</v>
+        <v>1.100302661056701E-3</v>
       </c>
       <c r="M4">
-        <v>2.6102082543709784E-5</v>
+        <v>-8.7757110840701574E-5</v>
       </c>
       <c r="N4">
-        <v>1.4441779640450439E-4</v>
+        <v>-1.4947585475790814E-3</v>
       </c>
       <c r="O4">
-        <v>-1.7894663167861979E-3</v>
+        <v>1.2088369009304446E-5</v>
       </c>
       <c r="P4">
-        <v>-1.2299244315679115E-3</v>
+        <v>-3.7145430702920255E-3</v>
       </c>
       <c r="Q4">
-        <v>8.4570820704380021E-4</v>
+        <v>9.8258554659475298E-4</v>
       </c>
       <c r="R4">
-        <v>7.0392566944827827E-4</v>
+        <v>3.3292275234410606E-3</v>
       </c>
       <c r="S4">
-        <v>9.9688721730346614E-5</v>
+        <v>1.3206990312926962E-4</v>
       </c>
       <c r="T4">
-        <v>-5.009227910631991E-4</v>
+        <v>-3.7923012566569328E-4</v>
       </c>
       <c r="U4">
-        <v>-1.1482362773312244E-3</v>
+        <v>-2.9596719659817005E-3</v>
       </c>
       <c r="V4">
-        <v>1.1254545305906362E-3</v>
+        <v>1.2881052067806157E-3</v>
       </c>
       <c r="W4">
-        <v>-3.3471972248961439E-5</v>
+        <v>5.6124109139208593E-4</v>
       </c>
       <c r="X4">
-        <v>2.2856607472792245E-4</v>
+        <v>-5.6944476809105203E-4</v>
       </c>
       <c r="Y4">
-        <v>3.1057699376862123E-4</v>
+        <v>8.8462643243483719E-4</v>
       </c>
       <c r="Z4">
-        <v>1.7767527515970575E-4</v>
+        <v>-3.6064803144921593E-5</v>
       </c>
       <c r="AA4">
-        <v>2.8429778853909923E-4</v>
+        <v>1.555712424833489E-4</v>
       </c>
       <c r="AB4">
-        <v>-1.5808479232049642E-5</v>
+        <v>-4.1240557598391076E-5</v>
       </c>
       <c r="AC4">
-        <v>2.3912491505732447E-4</v>
+        <v>-3.3106782533749848E-4</v>
       </c>
       <c r="AD4">
-        <v>3.1818351229789257E-4</v>
+        <v>1.9770032406867682E-4</v>
       </c>
       <c r="AE4">
-        <v>-1.2059508707464417E-2</v>
+        <v>-1.2387257461297358E-2</v>
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A5" s="4" t="s">
+      <c r="A5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="4">
-        <v>0.1844490687169042</v>
+      <c r="B5">
+        <v>-0.25374958465246789</v>
       </c>
       <c r="C5">
-        <v>-1.5599553235947998E-4</v>
+        <v>6.7063061460856388E-5</v>
       </c>
       <c r="D5">
-        <v>2.0828800479358259E-6</v>
+        <v>-1.2432081387031601E-7</v>
       </c>
       <c r="E5">
-        <v>1.1320569731069548E-2</v>
+        <v>1.5644749416402162E-2</v>
       </c>
       <c r="F5">
-        <v>1.2872111649297965E-2</v>
+        <v>1.7279542876207886E-2</v>
       </c>
       <c r="G5">
-        <v>1.2292005584855248E-2</v>
+        <v>1.6081353893827761E-2</v>
       </c>
       <c r="H5">
-        <v>1.2426352354062968E-2</v>
+        <v>1.6062702318711868E-2</v>
       </c>
       <c r="I5">
-        <v>7.9250022030465344E-5</v>
+        <v>-8.7380584592961679E-4</v>
       </c>
       <c r="J5">
-        <v>-3.7778947827987134E-5</v>
+        <v>1.042648556051197E-3</v>
       </c>
       <c r="K5">
-        <v>-3.2499269089043652E-5</v>
+        <v>-3.4233027565256941E-4</v>
       </c>
       <c r="L5">
-        <v>2.6041787162320654E-5</v>
+        <v>-1.5159552284008809E-4</v>
       </c>
       <c r="M5">
-        <v>-7.0223993073513079E-5</v>
+        <v>-4.144254055447839E-4</v>
       </c>
       <c r="N5">
-        <v>2.5516700505571251E-5</v>
+        <v>-1.7746651959421539E-3</v>
       </c>
       <c r="O5">
-        <v>-3.0266143440537893E-4</v>
+        <v>-7.1864096380589489E-4</v>
       </c>
       <c r="P5">
-        <v>-1.8572697416285927E-3</v>
+        <v>-3.5958768533381784E-3</v>
       </c>
       <c r="Q5">
-        <v>1.3745203024877932E-3</v>
+        <v>2.1904230782756311E-3</v>
       </c>
       <c r="R5">
-        <v>1.9093028696430976E-3</v>
+        <v>3.931381177573569E-3</v>
       </c>
       <c r="S5">
-        <v>-5.1143586603134314E-5</v>
+        <v>2.8870103684609013E-4</v>
       </c>
       <c r="T5">
-        <v>-3.9607453399681308E-4</v>
+        <v>-3.5511976392773979E-4</v>
       </c>
       <c r="U5">
-        <v>-7.9171013475877808E-4</v>
+        <v>3.2629992669071795E-3</v>
       </c>
       <c r="V5">
-        <v>1.7154813598231292E-3</v>
+        <v>1.8284194929131326E-3</v>
       </c>
       <c r="W5">
-        <v>4.3733593379901355E-4</v>
+        <v>6.4064025476095999E-4</v>
       </c>
       <c r="X5">
-        <v>2.2090543634875268E-4</v>
+        <v>-4.6659838500573642E-4</v>
       </c>
       <c r="Y5">
-        <v>2.9942339633353343E-4</v>
+        <v>1.1539576645116312E-3</v>
       </c>
       <c r="Z5">
-        <v>1.9853308174726752E-4</v>
+        <v>-2.7223485210811898E-4</v>
       </c>
       <c r="AA5">
-        <v>2.7598110523056212E-4</v>
+        <v>-1.6058912491110668E-4</v>
       </c>
       <c r="AB5">
-        <v>-1.4929545295904917E-5</v>
+        <v>7.8199851678291627E-5</v>
       </c>
       <c r="AC5">
-        <v>-3.279483099759891E-5</v>
+        <v>-3.8058554416651037E-4</v>
       </c>
       <c r="AD5">
-        <v>2.3388041275380824E-4</v>
+        <v>3.3909788902428654E-4</v>
       </c>
       <c r="AE5">
-        <v>-8.55532189017464E-3</v>
+        <v>-2.2905120743896279E-2</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A6" s="4" t="s">
+      <c r="A6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="4">
-        <v>0.27446037376774834</v>
+      <c r="B6">
+        <v>-0.21214793782289593</v>
       </c>
       <c r="C6">
-        <v>-2.6702735423156908E-4</v>
+        <v>-9.5887305326766703E-5</v>
       </c>
       <c r="D6">
-        <v>3.6712026487779582E-6</v>
+        <v>1.4494476693503668E-6</v>
       </c>
       <c r="E6">
-        <v>1.1280306269238073E-2</v>
+        <v>1.5527379691744369E-2</v>
       </c>
       <c r="F6">
-        <v>1.2292005584855248E-2</v>
+        <v>1.6081353893827761E-2</v>
       </c>
       <c r="G6">
-        <v>1.332486449366245E-2</v>
+        <v>1.7977515760037768E-2</v>
       </c>
       <c r="H6">
-        <v>1.2924970267410255E-2</v>
+        <v>1.7405567007719766E-2</v>
       </c>
       <c r="I6">
-        <v>1.9133704315979017E-4</v>
+        <v>-9.3296917241863478E-4</v>
       </c>
       <c r="J6">
-        <v>-9.2012767221337499E-5</v>
+        <v>8.3763844462088669E-4</v>
       </c>
       <c r="K6">
-        <v>7.6892589997919723E-4</v>
+        <v>-6.0811684368765242E-4</v>
       </c>
       <c r="L6">
-        <v>1.7683144426818096E-4</v>
+        <v>-2.4672873281724426E-4</v>
       </c>
       <c r="M6">
-        <v>3.0609222464490424E-5</v>
+        <v>-9.1678912365764087E-4</v>
       </c>
       <c r="N6">
-        <v>1.8268207282184663E-4</v>
+        <v>-2.0758450549380461E-3</v>
       </c>
       <c r="O6">
-        <v>-3.2937110831517818E-5</v>
+        <v>-1.8702395239357105E-4</v>
       </c>
       <c r="P6">
-        <v>-2.0252793650416588E-3</v>
+        <v>-3.1549629000851712E-3</v>
       </c>
       <c r="Q6">
-        <v>1.4044007377681978E-3</v>
+        <v>2.213426846800716E-3</v>
       </c>
       <c r="R6">
-        <v>2.2619350017223068E-3</v>
+        <v>4.2960331845344601E-3</v>
       </c>
       <c r="S6">
-        <v>7.4599790917970381E-5</v>
+        <v>4.6045447648880621E-5</v>
       </c>
       <c r="T6">
-        <v>-1.931234465921913E-4</v>
+        <v>-9.5926360009204389E-6</v>
       </c>
       <c r="U6">
-        <v>-8.0763066515607794E-4</v>
+        <v>-9.347311100260304E-3</v>
       </c>
       <c r="V6">
-        <v>1.8108383199628032E-3</v>
+        <v>2.8534725468392086E-3</v>
       </c>
       <c r="W6">
-        <v>7.7486338378691662E-4</v>
+        <v>1.7134888506063516E-3</v>
       </c>
       <c r="X6">
-        <v>1.4899534601413875E-4</v>
+        <v>5.7599084600067161E-4</v>
       </c>
       <c r="Y6">
-        <v>3.6094664196645993E-4</v>
+        <v>2.0178087705291104E-3</v>
       </c>
       <c r="Z6">
-        <v>2.2530322637951653E-4</v>
+        <v>3.111905074119673E-4</v>
       </c>
       <c r="AA6">
-        <v>3.9546046006957644E-4</v>
+        <v>5.2490679053886951E-4</v>
       </c>
       <c r="AB6">
-        <v>-2.6689480399168821E-6</v>
+        <v>-1.9824853210931477E-4</v>
       </c>
       <c r="AC6">
-        <v>1.3158211822331036E-5</v>
+        <v>-1.1234744616190403E-4</v>
       </c>
       <c r="AD6">
-        <v>1.7514425447485776E-4</v>
+        <v>-3.9797461241870326E-4</v>
       </c>
       <c r="AE6">
-        <v>-7.707975565897307E-3</v>
+        <v>9.8791132255200004E-4</v>
       </c>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A7" s="4" t="s">
+      <c r="A7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="4">
-        <v>0.37612250848583589</v>
+      <c r="B7">
+        <v>-3.794438309381995E-2</v>
       </c>
       <c r="C7">
-        <v>-2.6739376720805869E-4</v>
+        <v>9.1379723694169634E-5</v>
       </c>
       <c r="D7">
-        <v>3.4809970050741673E-6</v>
+        <v>-1.7199274866531414E-6</v>
       </c>
       <c r="E7">
-        <v>1.1290573524496765E-2</v>
+        <v>1.5418119334999938E-2</v>
       </c>
       <c r="F7">
-        <v>1.2426352354062968E-2</v>
+        <v>1.6062702318711868E-2</v>
       </c>
       <c r="G7">
-        <v>1.2924970267410255E-2</v>
+        <v>1.7405567007719766E-2</v>
       </c>
       <c r="H7">
-        <v>1.3839772299190145E-2</v>
+        <v>1.8747611972098236E-2</v>
       </c>
       <c r="I7">
-        <v>2.6026229509901243E-4</v>
+        <v>-8.3642587193154391E-4</v>
       </c>
       <c r="J7">
-        <v>-2.7422635542860996E-5</v>
+        <v>6.9468304637078327E-4</v>
       </c>
       <c r="K7">
-        <v>5.5371939317197961E-4</v>
+        <v>-6.4440130927274821E-4</v>
       </c>
       <c r="L7">
-        <v>2.0751314813649601E-4</v>
+        <v>-3.7285510514678197E-4</v>
       </c>
       <c r="M7">
-        <v>4.9513434686500497E-5</v>
+        <v>-1.1755351696067029E-3</v>
       </c>
       <c r="N7">
-        <v>1.4798977583223988E-4</v>
+        <v>-2.1963310811363417E-3</v>
       </c>
       <c r="O7">
-        <v>-2.0728071272302102E-4</v>
+        <v>2.6773540035407786E-5</v>
       </c>
       <c r="P7">
-        <v>-1.9193945033023304E-3</v>
+        <v>-2.8924257736682841E-3</v>
       </c>
       <c r="Q7">
-        <v>1.6537914542798754E-3</v>
+        <v>2.5474791375352645E-3</v>
       </c>
       <c r="R7">
-        <v>2.4738952248091104E-3</v>
+        <v>4.4855638125146794E-3</v>
       </c>
       <c r="S7">
-        <v>3.2980722929104134E-4</v>
+        <v>1.64285748659745E-4</v>
       </c>
       <c r="T7">
-        <v>4.4393048925213049E-5</v>
+        <v>3.5676189873261462E-4</v>
       </c>
       <c r="U7">
-        <v>-1.1885843689452662E-3</v>
+        <v>-1.0010428841263685E-2</v>
       </c>
       <c r="V7">
-        <v>1.7954571935368513E-3</v>
+        <v>3.0473936062167788E-3</v>
       </c>
       <c r="W7">
-        <v>8.621738419492082E-4</v>
+        <v>2.0052115667627927E-3</v>
       </c>
       <c r="X7">
-        <v>1.3861162955907996E-4</v>
+        <v>6.9347205352700454E-4</v>
       </c>
       <c r="Y7">
-        <v>2.8059981020544682E-4</v>
+        <v>2.275508788050011E-3</v>
       </c>
       <c r="Z7">
-        <v>2.605508110060199E-4</v>
+        <v>3.1228006393693979E-4</v>
       </c>
       <c r="AA7">
-        <v>4.0835041409025886E-4</v>
+        <v>7.0290194679995498E-4</v>
       </c>
       <c r="AB7">
-        <v>6.4342486495588409E-6</v>
+        <v>-2.275053647680643E-4</v>
       </c>
       <c r="AC7">
-        <v>5.1524792219336413E-5</v>
+        <v>-1.7836881509195371E-4</v>
       </c>
       <c r="AD7">
-        <v>1.6785572366683236E-4</v>
+        <v>-3.5256610842830015E-4</v>
       </c>
       <c r="AE7">
-        <v>-7.6562263933973307E-3</v>
+        <v>-7.1839709934884421E-4</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A8" s="4" t="s">
+      <c r="A8" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="4">
-        <v>-0.41306030413085165</v>
+      <c r="B8">
+        <v>-0.36878326658701727</v>
       </c>
       <c r="C8">
-        <v>-3.3654092924715977E-4</v>
+        <v>-3.0072084295433218E-4</v>
       </c>
       <c r="D8">
-        <v>4.9164130985844696E-6</v>
+        <v>4.0778520476240335E-6</v>
       </c>
       <c r="E8">
-        <v>6.7062584488728307E-5</v>
+        <v>-1.0753962923125821E-3</v>
       </c>
       <c r="F8">
-        <v>7.9250022030465344E-5</v>
+        <v>-8.7380584592961679E-4</v>
       </c>
       <c r="G8">
-        <v>1.9133704315979017E-4</v>
+        <v>-9.3296917241863478E-4</v>
       </c>
       <c r="H8">
-        <v>2.6026229509901243E-4</v>
+        <v>-8.3642587193154391E-4</v>
       </c>
       <c r="I8">
-        <v>7.0922058417701871E-4</v>
+        <v>1.1663985903579467E-3</v>
       </c>
       <c r="J8">
-        <v>-2.0170762753444441E-4</v>
+        <v>-3.1923651000350804E-4</v>
       </c>
       <c r="K8">
-        <v>7.2478399788315729E-4</v>
+        <v>1.3990869178578773E-4</v>
       </c>
       <c r="L8">
-        <v>4.4363445549170971E-5</v>
+        <v>1.6090711830415863E-4</v>
       </c>
       <c r="M8">
-        <v>1.4275141007548311E-6</v>
+        <v>1.0199937074932813E-4</v>
       </c>
       <c r="N8">
-        <v>1.522459078858048E-6</v>
+        <v>3.1896410036064138E-4</v>
       </c>
       <c r="O8">
-        <v>-3.7220929695892715E-4</v>
+        <v>-1.7523152869481523E-4</v>
       </c>
       <c r="P8">
-        <v>-2.2424052881128437E-4</v>
+        <v>-2.4439620415757412E-4</v>
       </c>
       <c r="Q8">
-        <v>5.0848613629210786E-4</v>
+        <v>4.7308982556767574E-4</v>
       </c>
       <c r="R8">
-        <v>4.071472439698908E-4</v>
+        <v>2.3158615364190312E-4</v>
       </c>
       <c r="S8">
-        <v>3.9436415991214404E-6</v>
+        <v>1.3562733082982104E-4</v>
       </c>
       <c r="T8">
-        <v>-1.2530241957560461E-4</v>
+        <v>5.6902944001849785E-5</v>
       </c>
       <c r="U8">
-        <v>-4.0315965918530892E-5</v>
+        <v>3.4933142166057168E-3</v>
       </c>
       <c r="V8">
-        <v>-2.3002156782194079E-4</v>
+        <v>-3.6181095557555679E-4</v>
       </c>
       <c r="W8">
-        <v>-5.3974580672169834E-5</v>
+        <v>-2.767875043506819E-4</v>
       </c>
       <c r="X8">
-        <v>1.596535067560154E-5</v>
+        <v>-7.7850032275234428E-5</v>
       </c>
       <c r="Y8">
-        <v>1.0238385191772319E-4</v>
+        <v>-2.9617804134391724E-4</v>
       </c>
       <c r="Z8">
-        <v>3.4609419491087924E-5</v>
+        <v>-2.7750551696720379E-4</v>
       </c>
       <c r="AA8">
-        <v>3.9438556723504873E-5</v>
+        <v>-2.165427260908937E-4</v>
       </c>
       <c r="AB8">
-        <v>-2.7214548413133252E-6</v>
+        <v>7.9762339600379759E-5</v>
       </c>
       <c r="AC8">
-        <v>-2.5578364481533339E-5</v>
+        <v>-4.8693203654902339E-5</v>
       </c>
       <c r="AD8">
-        <v>-5.9407444466610905E-5</v>
+        <v>-2.8823954779161811E-5</v>
       </c>
       <c r="AE8">
-        <v>4.6719183804137653E-3</v>
+        <v>-9.458810079688261E-4</v>
       </c>
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A9" s="4" t="s">
+      <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="4">
-        <v>0.56093378671650429</v>
+      <c r="B9">
+        <v>0.67214032524460321</v>
       </c>
       <c r="C9">
-        <v>9.8342213252174994E-5</v>
+        <v>-9.0818006520796378E-5</v>
       </c>
       <c r="D9">
-        <v>-8.4759990998648817E-7</v>
+        <v>2.1578858707211663E-6</v>
       </c>
       <c r="E9">
-        <v>1.9036617985941987E-5</v>
+        <v>1.0366554294107006E-3</v>
       </c>
       <c r="F9">
-        <v>-3.7778947827987134E-5</v>
+        <v>1.042648556051197E-3</v>
       </c>
       <c r="G9">
-        <v>-9.2012767221337499E-5</v>
+        <v>8.3763844462088669E-4</v>
       </c>
       <c r="H9">
-        <v>-2.7422635542860996E-5</v>
+        <v>6.9468304637078327E-4</v>
       </c>
       <c r="I9">
-        <v>-2.0170762753444441E-4</v>
+        <v>-3.1923651000350804E-4</v>
       </c>
       <c r="J9">
-        <v>1.0699542184820158E-3</v>
+        <v>1.5034699600935263E-3</v>
       </c>
       <c r="K9">
-        <v>-3.9693372344789049E-4</v>
+        <v>1.2342586240111832E-5</v>
       </c>
       <c r="L9">
-        <v>7.9312139127565699E-5</v>
+        <v>-3.9642029046557149E-5</v>
       </c>
       <c r="M9">
-        <v>2.0941614992615442E-5</v>
+        <v>-1.4671884627497078E-5</v>
       </c>
       <c r="N9">
-        <v>4.2723370883815132E-5</v>
+        <v>-2.323026270710485E-4</v>
       </c>
       <c r="O9">
-        <v>-3.1072209107085641E-5</v>
+        <v>-1.591639233410909E-4</v>
       </c>
       <c r="P9">
-        <v>2.099508191540614E-4</v>
+        <v>-2.2770236902859282E-5</v>
       </c>
       <c r="Q9">
-        <v>2.0846562536907653E-4</v>
+        <v>1.8110745063063219E-4</v>
       </c>
       <c r="R9">
-        <v>1.2881571186473638E-4</v>
+        <v>1.9570457331374391E-4</v>
       </c>
       <c r="S9">
-        <v>1.4029386085416724E-4</v>
+        <v>2.6685097109928075E-4</v>
       </c>
       <c r="T9">
-        <v>2.2074305865028154E-4</v>
+        <v>4.0082971452603519E-4</v>
       </c>
       <c r="U9">
-        <v>3.2994248329018538E-5</v>
+        <v>-3.1950436091474632E-3</v>
       </c>
       <c r="V9">
-        <v>-3.1131398564071446E-5</v>
+        <v>4.4284971095989549E-5</v>
       </c>
       <c r="W9">
-        <v>-1.514370799753645E-4</v>
+        <v>-1.1080150184194208E-4</v>
       </c>
       <c r="X9">
-        <v>-1.51395986420455E-5</v>
+        <v>-2.9735276442375153E-4</v>
       </c>
       <c r="Y9">
-        <v>-7.9660085159065244E-5</v>
+        <v>3.1027127734345765E-5</v>
       </c>
       <c r="Z9">
-        <v>5.1172868672602211E-5</v>
+        <v>-6.2188839705147776E-5</v>
       </c>
       <c r="AA9">
-        <v>-1.7265724705360424E-5</v>
+        <v>-1.6239261766208763E-4</v>
       </c>
       <c r="AB9">
-        <v>-2.7829571149668148E-6</v>
+        <v>-2.1941907255594692E-5</v>
       </c>
       <c r="AC9">
-        <v>-3.9288890784926135E-5</v>
+        <v>-2.9354741869922976E-4</v>
       </c>
       <c r="AD9">
-        <v>-3.1125863325718868E-5</v>
+        <v>-2.8384302803011391E-4</v>
       </c>
       <c r="AE9">
-        <v>-2.4581550854899849E-3</v>
+        <v>4.0779576794641205E-3</v>
       </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A10" s="4" t="s">
+      <c r="A10" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="4">
-        <v>-0.64712382259869561</v>
+      <c r="B10">
+        <v>7.7875191533664359E-2</v>
       </c>
       <c r="C10">
-        <v>-1.8877589968322069E-4</v>
+        <v>1.0206408574724157E-4</v>
       </c>
       <c r="D10">
-        <v>3.0324858947823705E-6</v>
+        <v>-1.4554829651541759E-6</v>
       </c>
       <c r="E10">
-        <v>2.8581898359109591E-4</v>
+        <v>-7.7187129409041037E-5</v>
       </c>
       <c r="F10">
-        <v>-3.2499269089043652E-5</v>
+        <v>-3.4233027565256941E-4</v>
       </c>
       <c r="G10">
-        <v>7.6892589997919723E-4</v>
+        <v>-6.0811684368765242E-4</v>
       </c>
       <c r="H10">
-        <v>5.5371939317197961E-4</v>
+        <v>-6.4440130927274821E-4</v>
       </c>
       <c r="I10">
-        <v>7.2478399788315729E-4</v>
+        <v>1.3990869178578773E-4</v>
       </c>
       <c r="J10">
-        <v>-3.9693372344789049E-4</v>
+        <v>1.2342586240111832E-5</v>
       </c>
       <c r="K10">
-        <v>0.11059377411863093</v>
+        <v>0.10246192973057192</v>
       </c>
       <c r="L10">
-        <v>8.3630292960545305E-2</v>
+        <v>7.9886352808894612E-2</v>
       </c>
       <c r="M10">
-        <v>8.3623036902625292E-2</v>
+        <v>7.9842090227712076E-2</v>
       </c>
       <c r="N10">
-        <v>8.3746692955021212E-2</v>
+        <v>7.9894971220947242E-2</v>
       </c>
       <c r="O10">
-        <v>-1.8266617968796389E-4</v>
+        <v>-3.7678059934378311E-4</v>
       </c>
       <c r="P10">
-        <v>-2.5036297542995606E-4</v>
+        <v>4.6101678998815288E-4</v>
       </c>
       <c r="Q10">
-        <v>1.9792630229049923E-4</v>
+        <v>2.9224530749283936E-4</v>
       </c>
       <c r="R10">
-        <v>4.0043684536892818E-4</v>
+        <v>-1.1255759961693763E-3</v>
       </c>
       <c r="S10">
-        <v>4.6918374592145543E-4</v>
+        <v>-1.1910415951903869E-4</v>
       </c>
       <c r="T10">
-        <v>5.5604009335982404E-5</v>
+        <v>2.4255833903196258E-4</v>
       </c>
       <c r="U10">
-        <v>5.5119593287239477E-4</v>
+        <v>-7.2647788215747244E-3</v>
       </c>
       <c r="V10">
-        <v>-1.0509328676614957E-4</v>
+        <v>-5.9380501088227011E-4</v>
       </c>
       <c r="W10">
-        <v>-1.7030843422933747E-4</v>
+        <v>-1.7200455675944748E-4</v>
       </c>
       <c r="X10">
-        <v>-3.8045096765947257E-4</v>
+        <v>1.6603513771593775E-4</v>
       </c>
       <c r="Y10">
-        <v>-2.4582271198870403E-4</v>
+        <v>-4.778326837388408E-4</v>
       </c>
       <c r="Z10">
-        <v>-1.284220570935005E-4</v>
+        <v>-3.8246733922961407E-4</v>
       </c>
       <c r="AA10">
-        <v>4.6902342506572204E-4</v>
+        <v>2.5723409530692409E-5</v>
       </c>
       <c r="AB10">
-        <v>-2.8285873803390448E-5</v>
+        <v>-1.2153932766847259E-4</v>
       </c>
       <c r="AC10">
-        <v>1.2965498805307535E-3</v>
+        <v>6.4573110388512628E-4</v>
       </c>
       <c r="AD10">
-        <v>1.7246407844620504E-4</v>
+        <v>-7.1332150796014036E-5</v>
       </c>
       <c r="AE10">
-        <v>-8.2742245904287581E-2</v>
+        <v>-6.9344512243916911E-2</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A11" s="4" t="s">
+      <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="4">
-        <v>-0.55221004929509876</v>
+      <c r="B11">
+        <v>0.14500304335468325</v>
       </c>
       <c r="C11">
-        <v>-1.0975709844830445E-4</v>
+        <v>1.1566475225018719E-4</v>
       </c>
       <c r="D11">
-        <v>2.2771119802513846E-6</v>
+        <v>-1.5482169949105717E-6</v>
       </c>
       <c r="E11">
-        <v>1.9187935253608566E-4</v>
+        <v>1.100302661056701E-3</v>
       </c>
       <c r="F11">
-        <v>2.6041787162320654E-5</v>
+        <v>-1.5159552284008809E-4</v>
       </c>
       <c r="G11">
-        <v>1.7683144426818096E-4</v>
+        <v>-2.4672873281724426E-4</v>
       </c>
       <c r="H11">
-        <v>2.0751314813649601E-4</v>
+        <v>-3.7285510514678197E-4</v>
       </c>
       <c r="I11">
-        <v>4.4363445549170971E-5</v>
+        <v>1.6090711830415863E-4</v>
       </c>
       <c r="J11">
-        <v>7.9312139127565699E-5</v>
+        <v>-3.9642029046557149E-5</v>
       </c>
       <c r="K11">
-        <v>8.3630292960545305E-2</v>
+        <v>7.9886352808894612E-2</v>
       </c>
       <c r="L11">
-        <v>8.617942676225436E-2</v>
+        <v>8.4401554231552184E-2</v>
       </c>
       <c r="M11">
-        <v>8.4019119390448399E-2</v>
+        <v>7.9900025866150332E-2</v>
       </c>
       <c r="N11">
-        <v>8.4076260911171707E-2</v>
+        <v>7.9858906155957976E-2</v>
       </c>
       <c r="O11">
-        <v>9.5346709301363797E-6</v>
+        <v>-8.6859376383478099E-4</v>
       </c>
       <c r="P11">
-        <v>3.7303760612540648E-5</v>
+        <v>6.8685794684207602E-4</v>
       </c>
       <c r="Q11">
-        <v>-4.4398154379718391E-5</v>
+        <v>7.1041138971651707E-4</v>
       </c>
       <c r="R11">
-        <v>1.6280482176972422E-4</v>
+        <v>-8.6346397203709152E-4</v>
       </c>
       <c r="S11">
-        <v>4.2441989283114841E-5</v>
+        <v>-2.2862063244203507E-4</v>
       </c>
       <c r="T11">
-        <v>2.5658339404524035E-4</v>
+        <v>1.7847483114818985E-4</v>
       </c>
       <c r="U11">
-        <v>-1.6059617628885747E-4</v>
+        <v>-3.649038641633684E-3</v>
       </c>
       <c r="V11">
-        <v>3.7888829995916251E-4</v>
+        <v>-3.1392029688528944E-4</v>
       </c>
       <c r="W11">
-        <v>4.0183811021562987E-4</v>
+        <v>6.3305338590252669E-5</v>
       </c>
       <c r="X11">
-        <v>-3.7671397780852066E-4</v>
+        <v>7.2134580263658044E-5</v>
       </c>
       <c r="Y11">
-        <v>-3.4137581956191192E-4</v>
+        <v>-4.3427722434931371E-4</v>
       </c>
       <c r="Z11">
-        <v>-1.2230621992551528E-4</v>
+        <v>-3.3983709615911795E-4</v>
       </c>
       <c r="AA11">
-        <v>-1.0161682224577289E-4</v>
+        <v>-1.5114739733154692E-4</v>
       </c>
       <c r="AB11">
-        <v>-1.3468760293948025E-5</v>
+        <v>-6.3188053292702329E-5</v>
       </c>
       <c r="AC11">
-        <v>-6.8579148196939999E-5</v>
+        <v>1.084405486169622E-3</v>
       </c>
       <c r="AD11">
-        <v>-2.1924498427777772E-5</v>
+        <v>8.4224755973066195E-5</v>
       </c>
       <c r="AE11">
-        <v>-8.2753910604096759E-2</v>
+        <v>-7.592401252361336E-2</v>
       </c>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A12" s="4" t="s">
+      <c r="A12" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="4">
-        <v>-0.41366978380732133</v>
+      <c r="B12">
+        <v>0.24475747577542964</v>
       </c>
       <c r="C12">
-        <v>-8.5185570430833853E-5</v>
+        <v>-4.0148122286011445E-5</v>
       </c>
       <c r="D12">
-        <v>2.0995616541072575E-6</v>
+        <v>9.6509726436080608E-7</v>
       </c>
       <c r="E12">
-        <v>2.6102082543709784E-5</v>
+        <v>-8.7757110840701574E-5</v>
       </c>
       <c r="F12">
-        <v>-7.0223993073513079E-5</v>
+        <v>-4.144254055447839E-4</v>
       </c>
       <c r="G12">
-        <v>3.0609222464490424E-5</v>
+        <v>-9.1678912365764087E-4</v>
       </c>
       <c r="H12">
-        <v>4.9513434686500497E-5</v>
+        <v>-1.1755351696067029E-3</v>
       </c>
       <c r="I12">
-        <v>1.4275141007548311E-6</v>
+        <v>1.0199937074932813E-4</v>
       </c>
       <c r="J12">
-        <v>2.0941614992615442E-5</v>
+        <v>-1.4671884627497078E-5</v>
       </c>
       <c r="K12">
-        <v>8.3623036902625292E-2</v>
+        <v>7.9842090227712076E-2</v>
       </c>
       <c r="L12">
-        <v>8.4019119390448399E-2</v>
+        <v>7.9900025866150332E-2</v>
       </c>
       <c r="M12">
-        <v>8.4511826872225915E-2</v>
+        <v>8.0462487804507321E-2</v>
       </c>
       <c r="N12">
-        <v>8.4288846745117718E-2</v>
+        <v>8.0004105150030841E-2</v>
       </c>
       <c r="O12">
-        <v>1.1969336146926135E-4</v>
+        <v>-9.1941523039774237E-4</v>
       </c>
       <c r="P12">
-        <v>5.0855648844080198E-4</v>
+        <v>3.6727462076713291E-4</v>
       </c>
       <c r="Q12">
-        <v>-8.549177615355813E-5</v>
+        <v>6.1208162672234633E-4</v>
       </c>
       <c r="R12">
-        <v>-7.739434985204463E-5</v>
+        <v>-8.728663974081341E-4</v>
       </c>
       <c r="S12">
-        <v>1.113668778462131E-4</v>
+        <v>4.2384003691629812E-5</v>
       </c>
       <c r="T12">
-        <v>5.1059293718817671E-4</v>
+        <v>3.7725084422883873E-4</v>
       </c>
       <c r="U12">
-        <v>7.3705097809739772E-4</v>
+        <v>-2.9094610916571284E-3</v>
       </c>
       <c r="V12">
-        <v>2.5820894272164316E-4</v>
+        <v>-6.1070456127521044E-4</v>
       </c>
       <c r="W12">
-        <v>4.4745943156195706E-4</v>
+        <v>-1.5116710570581976E-4</v>
       </c>
       <c r="X12">
-        <v>-4.6427709508903119E-4</v>
+        <v>-3.8423601706332605E-4</v>
       </c>
       <c r="Y12">
-        <v>-1.9277684255405948E-4</v>
+        <v>-6.121932368545191E-4</v>
       </c>
       <c r="Z12">
-        <v>-1.3906646043800389E-4</v>
+        <v>-5.6821633514136938E-4</v>
       </c>
       <c r="AA12">
-        <v>-4.9608189989342431E-5</v>
+        <v>-3.9098676380741604E-4</v>
       </c>
       <c r="AB12">
-        <v>-3.8728019827620447E-5</v>
+        <v>-3.1311804414090039E-5</v>
       </c>
       <c r="AC12">
-        <v>-5.9849585982117703E-5</v>
+        <v>7.1781241283169067E-4</v>
       </c>
       <c r="AD12">
-        <v>1.2623628609969434E-4</v>
+        <v>1.2550409944924509E-4</v>
       </c>
       <c r="AE12">
-        <v>-8.4244609024092143E-2</v>
+        <v>-7.4408123300112816E-2</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A13" s="4" t="s">
+      <c r="A13" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="4">
-        <v>-0.44881433206752941</v>
+      <c r="B13">
+        <v>0.22931572616828355</v>
       </c>
       <c r="C13">
-        <v>-1.3499536097145645E-4</v>
+        <v>-8.9329145078764077E-5</v>
       </c>
       <c r="D13">
-        <v>3.0967256168015677E-6</v>
+        <v>1.4300579061547161E-6</v>
       </c>
       <c r="E13">
-        <v>1.4441779640450439E-4</v>
+        <v>-1.4947585475790814E-3</v>
       </c>
       <c r="F13">
-        <v>2.5516700505571251E-5</v>
+        <v>-1.7746651959421539E-3</v>
       </c>
       <c r="G13">
-        <v>1.8268207282184663E-4</v>
+        <v>-2.0758450549380461E-3</v>
       </c>
       <c r="H13">
-        <v>1.4798977583223988E-4</v>
+        <v>-2.1963310811363417E-3</v>
       </c>
       <c r="I13">
-        <v>1.522459078858048E-6</v>
+        <v>3.1896410036064138E-4</v>
       </c>
       <c r="J13">
-        <v>4.2723370883815132E-5</v>
+        <v>-2.323026270710485E-4</v>
       </c>
       <c r="K13">
-        <v>8.3746692955021212E-2</v>
+        <v>7.9894971220947242E-2</v>
       </c>
       <c r="L13">
-        <v>8.4076260911171707E-2</v>
+        <v>7.9858906155957976E-2</v>
       </c>
       <c r="M13">
-        <v>8.4288846745117718E-2</v>
+        <v>8.0004105150030841E-2</v>
       </c>
       <c r="N13">
-        <v>8.5234064808457105E-2</v>
+        <v>8.1641485599922209E-2</v>
       </c>
       <c r="O13">
-        <v>4.7484290588423184E-4</v>
+        <v>-8.1412246595042453E-4</v>
       </c>
       <c r="P13">
-        <v>5.9352234694221712E-4</v>
+        <v>4.0464487793898107E-4</v>
       </c>
       <c r="Q13">
-        <v>-3.7995597374610585E-4</v>
+        <v>6.6901163816584109E-4</v>
       </c>
       <c r="R13">
-        <v>5.2295763002838808E-5</v>
+        <v>-8.4072254684584499E-4</v>
       </c>
       <c r="S13">
-        <v>1.1437322066732022E-4</v>
+        <v>-2.5038062205174488E-4</v>
       </c>
       <c r="T13">
-        <v>5.7813511922817987E-4</v>
+        <v>3.0245107304069374E-4</v>
       </c>
       <c r="U13">
-        <v>5.5518875917112687E-4</v>
+        <v>-4.2623579171752191E-3</v>
       </c>
       <c r="V13">
-        <v>2.4249225575666625E-4</v>
+        <v>-7.1168020374343111E-4</v>
       </c>
       <c r="W13">
-        <v>4.9592163070215529E-4</v>
+        <v>-6.0703632047888478E-5</v>
       </c>
       <c r="X13">
-        <v>-3.9430563060456614E-4</v>
+        <v>-7.0866272852798673E-5</v>
       </c>
       <c r="Y13">
-        <v>-1.7100302444384395E-4</v>
+        <v>-6.9105148763527746E-4</v>
       </c>
       <c r="Z13">
-        <v>-1.4266392760561245E-4</v>
+        <v>-3.3076199473364154E-4</v>
       </c>
       <c r="AA13">
-        <v>3.8489258457458618E-5</v>
+        <v>-1.8219403422939373E-4</v>
       </c>
       <c r="AB13">
-        <v>-3.7190050698999972E-5</v>
+        <v>-7.879956687860401E-5</v>
       </c>
       <c r="AC13">
-        <v>-1.1601445814387462E-4</v>
+        <v>9.289849170115716E-4</v>
       </c>
       <c r="AD13">
-        <v>1.4057615879197946E-4</v>
+        <v>-1.0482830196222558E-5</v>
       </c>
       <c r="AE13">
-        <v>-8.3793811011936059E-2</v>
+        <v>-6.980181834357313E-2</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A14" s="4" t="s">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="4">
-        <v>-1.356913036515945</v>
+      <c r="B14">
+        <v>-0.88495250152528759</v>
       </c>
       <c r="C14">
-        <v>7.6912382475424756E-5</v>
+        <v>-3.0777543329596566E-4</v>
       </c>
       <c r="D14">
-        <v>-1.2798079003760058E-6</v>
+        <v>3.7347654422265314E-6</v>
       </c>
       <c r="E14">
-        <v>-1.7894663167861979E-3</v>
+        <v>1.2088369009304446E-5</v>
       </c>
       <c r="F14">
-        <v>-3.0266143440537893E-4</v>
+        <v>-7.1864096380589489E-4</v>
       </c>
       <c r="G14">
-        <v>-3.2937110831517818E-5</v>
+        <v>-1.8702395239357105E-4</v>
       </c>
       <c r="H14">
-        <v>-2.0728071272302102E-4</v>
+        <v>2.6773540035407786E-5</v>
       </c>
       <c r="I14">
-        <v>-3.7220929695892715E-4</v>
+        <v>-1.7523152869481523E-4</v>
       </c>
       <c r="J14">
-        <v>-3.1072209107085641E-5</v>
+        <v>-1.591639233410909E-4</v>
       </c>
       <c r="K14">
-        <v>-1.8266617968796389E-4</v>
+        <v>-3.7678059934378311E-4</v>
       </c>
       <c r="L14">
-        <v>9.5346709301363797E-6</v>
+        <v>-8.6859376383478099E-4</v>
       </c>
       <c r="M14">
-        <v>1.1969336146926135E-4</v>
+        <v>-9.1941523039774237E-4</v>
       </c>
       <c r="N14">
-        <v>4.7484290588423184E-4</v>
+        <v>-8.1412246595042453E-4</v>
       </c>
       <c r="O14">
-        <v>3.1729585625160643E-2</v>
+        <v>2.8576406519526577E-2</v>
       </c>
       <c r="P14">
-        <v>6.6023205155492934E-3</v>
+        <v>2.7762420239396601E-3</v>
       </c>
       <c r="Q14">
-        <v>-2.7469863201270164E-2</v>
+        <v>-2.319284804840073E-2</v>
       </c>
       <c r="R14">
-        <v>-4.7857464266051588E-3</v>
+        <v>-2.2648935501520585E-3</v>
       </c>
       <c r="S14">
-        <v>-2.1134127580801423E-6</v>
+        <v>-5.434939854039476E-4</v>
       </c>
       <c r="T14">
-        <v>4.811464463765682E-4</v>
+        <v>-1.4841064432457267E-4</v>
       </c>
       <c r="U14">
-        <v>-5.0795982176589762E-4</v>
+        <v>-1.0375994015841185E-2</v>
       </c>
       <c r="V14">
-        <v>6.9032131691097189E-4</v>
+        <v>6.2335694107264845E-4</v>
       </c>
       <c r="W14">
-        <v>1.4831380963284302E-4</v>
+        <v>4.7680745231862341E-4</v>
       </c>
       <c r="X14">
-        <v>7.6876093061210106E-5</v>
+        <v>-6.0251583119956499E-5</v>
       </c>
       <c r="Y14">
-        <v>1.0344903868390441E-4</v>
+        <v>2.975705552297446E-4</v>
       </c>
       <c r="Z14">
-        <v>8.3212268812885487E-5</v>
+        <v>2.5410061215240445E-4</v>
       </c>
       <c r="AA14">
-        <v>4.962905437433277E-5</v>
+        <v>2.6284742542824436E-4</v>
       </c>
       <c r="AB14">
-        <v>4.1569522667938513E-5</v>
+        <v>-2.2960068732225786E-4</v>
       </c>
       <c r="AC14">
-        <v>-5.2681368138991151E-4</v>
+        <v>-2.0857481001030124E-5</v>
       </c>
       <c r="AD14">
-        <v>-1.1693663405852828E-4</v>
+        <v>-3.2755124765183712E-4</v>
       </c>
       <c r="AE14">
-        <v>-6.2254617512547822E-4</v>
+        <v>2.5008630614879075E-2</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A15" s="4" t="s">
+      <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4">
-        <v>-0.91765994945200646</v>
+      <c r="B15">
+        <v>-0.60103951249965404</v>
       </c>
       <c r="C15">
-        <v>-1.1692880680639565E-4</v>
+        <v>1.7080749835791595E-5</v>
       </c>
       <c r="D15">
-        <v>2.0231536991994901E-6</v>
+        <v>-4.9467523507792E-7</v>
       </c>
       <c r="E15">
-        <v>-1.2299244315679115E-3</v>
+        <v>-3.7145430702920255E-3</v>
       </c>
       <c r="F15">
-        <v>-1.8572697416285927E-3</v>
+        <v>-3.5958768533381784E-3</v>
       </c>
       <c r="G15">
-        <v>-2.0252793650416588E-3</v>
+        <v>-3.1549629000851712E-3</v>
       </c>
       <c r="H15">
-        <v>-1.9193945033023304E-3</v>
+        <v>-2.8924257736682841E-3</v>
       </c>
       <c r="I15">
-        <v>-2.2424052881128437E-4</v>
+        <v>-2.4439620415757412E-4</v>
       </c>
       <c r="J15">
-        <v>2.099508191540614E-4</v>
+        <v>-2.2770236902859282E-5</v>
       </c>
       <c r="K15">
-        <v>-2.5036297542995606E-4</v>
+        <v>4.6101678998815288E-4</v>
       </c>
       <c r="L15">
-        <v>3.7303760612540648E-5</v>
+        <v>6.8685794684207602E-4</v>
       </c>
       <c r="M15">
-        <v>5.0855648844080198E-4</v>
+        <v>3.6727462076713291E-4</v>
       </c>
       <c r="N15">
-        <v>5.9352234694221712E-4</v>
+        <v>4.0464487793898107E-4</v>
       </c>
       <c r="O15">
-        <v>6.6023205155492934E-3</v>
+        <v>2.7762420239396601E-3</v>
       </c>
       <c r="P15">
-        <v>2.205402467012002E-2</v>
+        <v>2.6367085456375762E-2</v>
       </c>
       <c r="Q15">
-        <v>-7.0301688258032312E-3</v>
+        <v>-2.6094053066738425E-3</v>
       </c>
       <c r="R15">
-        <v>-1.7580472239878811E-2</v>
+        <v>-2.2258292865243431E-2</v>
       </c>
       <c r="S15">
-        <v>-1.32841498703681E-4</v>
+        <v>-4.0603738631635514E-4</v>
       </c>
       <c r="T15">
-        <v>4.8786060506086958E-4</v>
+        <v>-2.0658737129131653E-4</v>
       </c>
       <c r="U15">
-        <v>2.1220970524371673E-3</v>
+        <v>-7.998476587633821E-3</v>
       </c>
       <c r="V15">
-        <v>4.3644292906844982E-5</v>
+        <v>-5.9864412779825436E-4</v>
       </c>
       <c r="W15">
-        <v>2.7818894293340899E-4</v>
+        <v>5.812671467913188E-4</v>
       </c>
       <c r="X15">
-        <v>-9.6934724572757524E-5</v>
+        <v>2.2828525415892866E-4</v>
       </c>
       <c r="Y15">
-        <v>4.9287291610111998E-4</v>
+        <v>5.1378747704251739E-5</v>
       </c>
       <c r="Z15">
-        <v>2.1397395422366526E-4</v>
+        <v>3.4452728579310258E-4</v>
       </c>
       <c r="AA15">
-        <v>-4.8228911015247774E-6</v>
+        <v>1.6895230994670891E-4</v>
       </c>
       <c r="AB15">
-        <v>-3.8323392250187401E-5</v>
+        <v>-1.8890471060084807E-4</v>
       </c>
       <c r="AC15">
-        <v>1.7784775603164904E-4</v>
+        <v>5.5571748364532448E-4</v>
       </c>
       <c r="AD15">
-        <v>1.2564404886540901E-4</v>
+        <v>-3.36103046794762E-4</v>
       </c>
       <c r="AE15">
-        <v>8.6616340823723252E-4</v>
+        <v>1.6504489093138681E-2</v>
       </c>
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A16" s="4" t="s">
+      <c r="A16" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="4">
-        <v>1.2195717217396631</v>
+      <c r="B16">
+        <v>0.80427320195749852</v>
       </c>
       <c r="C16">
-        <v>-7.3303706793806898E-5</v>
+        <v>1.520296086144089E-4</v>
       </c>
       <c r="D16">
-        <v>1.7874509792603665E-6</v>
+        <v>-1.6566145337345119E-6</v>
       </c>
       <c r="E16">
-        <v>8.4570820704380021E-4</v>
+        <v>9.8258554659475298E-4</v>
       </c>
       <c r="F16">
-        <v>1.3745203024877932E-3</v>
+        <v>2.1904230782756311E-3</v>
       </c>
       <c r="G16">
-        <v>1.4044007377681978E-3</v>
+        <v>2.213426846800716E-3</v>
       </c>
       <c r="H16">
-        <v>1.6537914542798754E-3</v>
+        <v>2.5474791375352645E-3</v>
       </c>
       <c r="I16">
-        <v>5.0848613629210786E-4</v>
+        <v>4.7308982556767574E-4</v>
       </c>
       <c r="J16">
-        <v>2.0846562536907653E-4</v>
+        <v>1.8110745063063219E-4</v>
       </c>
       <c r="K16">
-        <v>1.9792630229049923E-4</v>
+        <v>2.9224530749283936E-4</v>
       </c>
       <c r="L16">
-        <v>-4.4398154379718391E-5</v>
+        <v>7.1041138971651707E-4</v>
       </c>
       <c r="M16">
-        <v>-8.549177615355813E-5</v>
+        <v>6.1208162672234633E-4</v>
       </c>
       <c r="N16">
-        <v>-3.7995597374610585E-4</v>
+        <v>6.6901163816584109E-4</v>
       </c>
       <c r="O16">
-        <v>-2.7469863201270164E-2</v>
+        <v>-2.319284804840073E-2</v>
       </c>
       <c r="P16">
-        <v>-7.0301688258032312E-3</v>
+        <v>-2.6094053066738425E-3</v>
       </c>
       <c r="Q16">
-        <v>2.8221062299334711E-2</v>
+        <v>2.4385032493327359E-2</v>
       </c>
       <c r="R16">
-        <v>5.8929398015794702E-3</v>
+        <v>3.1561818223486142E-3</v>
       </c>
       <c r="S16">
-        <v>-4.0754449678660542E-5</v>
+        <v>3.0415089520170356E-4</v>
       </c>
       <c r="T16">
-        <v>-7.2425620442973676E-4</v>
+        <v>3.0109542111242957E-4</v>
       </c>
       <c r="U16">
-        <v>-2.9147874716058033E-4</v>
+        <v>8.82665705467163E-3</v>
       </c>
       <c r="V16">
-        <v>-1.4736186988996832E-3</v>
+        <v>-6.9298365517534745E-4</v>
       </c>
       <c r="W16">
-        <v>1.6550412430280532E-4</v>
+        <v>3.7250565870342815E-4</v>
       </c>
       <c r="X16">
-        <v>-2.661655520219098E-4</v>
+        <v>8.0731490063672487E-5</v>
       </c>
       <c r="Y16">
-        <v>-1.5986730426279362E-4</v>
+        <v>-6.399401024035755E-5</v>
       </c>
       <c r="Z16">
-        <v>-8.3156147322452931E-5</v>
+        <v>-2.9044001037349838E-4</v>
       </c>
       <c r="AA16">
-        <v>-5.6907486115411382E-5</v>
+        <v>-2.877600456760495E-4</v>
       </c>
       <c r="AB16">
-        <v>-3.8230551777755741E-5</v>
+        <v>1.6316875023124995E-4</v>
       </c>
       <c r="AC16">
-        <v>4.545165394622421E-4</v>
+        <v>3.222092623969895E-4</v>
       </c>
       <c r="AD16">
-        <v>-8.3217073198970336E-6</v>
+        <v>1.978664787983278E-4</v>
       </c>
       <c r="AE16">
-        <v>-8.4558287762910578E-4</v>
+        <v>-2.1883668073604076E-2</v>
       </c>
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A17" s="4" t="s">
+      <c r="A17" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="4">
-        <v>0.61948063204069437</v>
+      <c r="B17">
+        <v>0.27142996688325505</v>
       </c>
       <c r="C17">
-        <v>-2.5130572391913238E-4</v>
+        <v>-4.5032176654757634E-5</v>
       </c>
       <c r="D17">
-        <v>3.9857705274844041E-6</v>
+        <v>6.1326581762181589E-7</v>
       </c>
       <c r="E17">
-        <v>7.0392566944827827E-4</v>
+        <v>3.3292275234410606E-3</v>
       </c>
       <c r="F17">
-        <v>1.9093028696430976E-3</v>
+        <v>3.931381177573569E-3</v>
       </c>
       <c r="G17">
-        <v>2.2619350017223068E-3</v>
+        <v>4.2960331845344601E-3</v>
       </c>
       <c r="H17">
-        <v>2.4738952248091104E-3</v>
+        <v>4.4855638125146794E-3</v>
       </c>
       <c r="I17">
-        <v>4.071472439698908E-4</v>
+        <v>2.3158615364190312E-4</v>
       </c>
       <c r="J17">
-        <v>1.2881571186473638E-4</v>
+        <v>1.9570457331374391E-4</v>
       </c>
       <c r="K17">
-        <v>4.0043684536892818E-4</v>
+        <v>-1.1255759961693763E-3</v>
       </c>
       <c r="L17">
-        <v>1.6280482176972422E-4</v>
+        <v>-8.6346397203709152E-4</v>
       </c>
       <c r="M17">
-        <v>-7.739434985204463E-5</v>
+        <v>-8.728663974081341E-4</v>
       </c>
       <c r="N17">
-        <v>5.2295763002838808E-5</v>
+        <v>-8.4072254684584499E-4</v>
       </c>
       <c r="O17">
-        <v>-4.7857464266051588E-3</v>
+        <v>-2.2648935501520585E-3</v>
       </c>
       <c r="P17">
-        <v>-1.7580472239878811E-2</v>
+        <v>-2.2258292865243431E-2</v>
       </c>
       <c r="Q17">
-        <v>5.8929398015794702E-3</v>
+        <v>3.1561818223486142E-3</v>
       </c>
       <c r="R17">
-        <v>1.8414443920753601E-2</v>
+        <v>2.4500604760612905E-2</v>
       </c>
       <c r="S17">
-        <v>6.9101004117114772E-5</v>
+        <v>2.3453967674091697E-4</v>
       </c>
       <c r="T17">
-        <v>-3.7907013253733887E-4</v>
+        <v>2.3332758907138713E-4</v>
       </c>
       <c r="U17">
-        <v>-2.5543451940962122E-3</v>
+        <v>4.0235680416472949E-3</v>
       </c>
       <c r="V17">
-        <v>-1.8369318955659765E-4</v>
+        <v>1.3423975894431648E-3</v>
       </c>
       <c r="W17">
-        <v>-6.4661622260776255E-6</v>
+        <v>4.2163652572025463E-4</v>
       </c>
       <c r="X17">
-        <v>1.7546977267600099E-4</v>
+        <v>-1.1991082457825809E-4</v>
       </c>
       <c r="Y17">
-        <v>-2.2846398251503505E-4</v>
+        <v>4.3593541650084958E-4</v>
       </c>
       <c r="Z17">
-        <v>-8.2324881837983325E-5</v>
+        <v>4.08985385420748E-5</v>
       </c>
       <c r="AA17">
-        <v>1.7121583925899119E-4</v>
+        <v>2.5207197076730983E-5</v>
       </c>
       <c r="AB17">
-        <v>3.086857548289209E-5</v>
+        <v>7.5724639217917417E-5</v>
       </c>
       <c r="AC17">
-        <v>-3.1174316931970438E-4</v>
+        <v>-4.4206742426121902E-4</v>
       </c>
       <c r="AD17">
-        <v>-2.4049389922529464E-4</v>
+        <v>7.7905155236683771E-5</v>
       </c>
       <c r="AE17">
-        <v>3.7602632527530353E-3</v>
+        <v>-1.0053438042088594E-2</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A18" s="4" t="s">
+      <c r="A18" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="4">
-        <v>-0.1205474725943646</v>
+      <c r="B18">
+        <v>-0.28530008667805085</v>
       </c>
       <c r="C18">
-        <v>1.9243435626443449E-4</v>
+        <v>3.540702064387842E-5</v>
       </c>
       <c r="D18">
-        <v>-2.8319923634328983E-6</v>
+        <v>-9.1955951857247437E-9</v>
       </c>
       <c r="E18">
-        <v>9.9688721730346614E-5</v>
+        <v>1.3206990312926962E-4</v>
       </c>
       <c r="F18">
-        <v>-5.1143586603134314E-5</v>
+        <v>2.8870103684609013E-4</v>
       </c>
       <c r="G18">
-        <v>7.4599790917970381E-5</v>
+        <v>4.6045447648880621E-5</v>
       </c>
       <c r="H18">
-        <v>3.2980722929104134E-4</v>
+        <v>1.64285748659745E-4</v>
       </c>
       <c r="I18">
-        <v>3.9436415991214404E-6</v>
+        <v>1.3562733082982104E-4</v>
       </c>
       <c r="J18">
-        <v>1.4029386085416724E-4</v>
+        <v>2.6685097109928075E-4</v>
       </c>
       <c r="K18">
-        <v>4.6918374592145543E-4</v>
+        <v>-1.1910415951903869E-4</v>
       </c>
       <c r="L18">
-        <v>4.2441989283114841E-5</v>
+        <v>-2.2862063244203507E-4</v>
       </c>
       <c r="M18">
-        <v>1.113668778462131E-4</v>
+        <v>4.2384003691629812E-5</v>
       </c>
       <c r="N18">
-        <v>1.1437322066732022E-4</v>
+        <v>-2.5038062205174488E-4</v>
       </c>
       <c r="O18">
-        <v>-2.1134127580801423E-6</v>
+        <v>-5.434939854039476E-4</v>
       </c>
       <c r="P18">
-        <v>-1.32841498703681E-4</v>
+        <v>-4.0603738631635514E-4</v>
       </c>
       <c r="Q18">
-        <v>-4.0754449678660542E-5</v>
+        <v>3.0415089520170356E-4</v>
       </c>
       <c r="R18">
-        <v>6.9101004117114772E-5</v>
+        <v>2.3453967674091697E-4</v>
       </c>
       <c r="S18">
-        <v>1.0828448908609188E-3</v>
+        <v>1.9210799163307988E-3</v>
       </c>
       <c r="T18">
-        <v>8.152753097305799E-4</v>
+        <v>1.2483683570379677E-3</v>
       </c>
       <c r="U18">
-        <v>-5.0083306979949518E-6</v>
+        <v>7.9949883265242883E-3</v>
       </c>
       <c r="V18">
-        <v>1.9592037078065437E-4</v>
+        <v>6.1913401883952578E-5</v>
       </c>
       <c r="W18">
-        <v>-1.3280603289883791E-4</v>
+        <v>-3.6821600525828208E-4</v>
       </c>
       <c r="X18">
-        <v>-1.0403971901812124E-4</v>
+        <v>-4.6164450322705355E-4</v>
       </c>
       <c r="Y18">
-        <v>-5.4826601102152367E-5</v>
+        <v>-2.4991452807371318E-4</v>
       </c>
       <c r="Z18">
-        <v>-2.3388965619314977E-5</v>
+        <v>-3.1266888160362202E-4</v>
       </c>
       <c r="AA18">
-        <v>4.2485836602178115E-5</v>
+        <v>-3.3986133414734814E-4</v>
       </c>
       <c r="AB18">
-        <v>1.5451025931629641E-5</v>
+        <v>1.9454093844275947E-4</v>
       </c>
       <c r="AC18">
-        <v>1.1634006715949784E-4</v>
+        <v>-1.3531950853782064E-4</v>
       </c>
       <c r="AD18">
-        <v>1.2973870902276401E-6</v>
+        <v>4.2491279157220584E-5</v>
       </c>
       <c r="AE18">
-        <v>-4.2793830195181314E-3</v>
+        <v>-1.6196901215115495E-2</v>
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A19" s="4" t="s">
+      <c r="A19" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="4">
-        <v>5.9088557073164148E-2</v>
+      <c r="B19">
+        <v>-0.41909387824518635</v>
       </c>
       <c r="C19">
-        <v>4.4902128542772526E-4</v>
+        <v>1.5759634054272626E-4</v>
       </c>
       <c r="D19">
-        <v>-6.4012366243920116E-6</v>
+        <v>-1.9322631231452825E-6</v>
       </c>
       <c r="E19">
-        <v>-5.009227910631991E-4</v>
+        <v>-3.7923012566569328E-4</v>
       </c>
       <c r="F19">
-        <v>-3.9607453399681308E-4</v>
+        <v>-3.5511976392773979E-4</v>
       </c>
       <c r="G19">
-        <v>-1.931234465921913E-4</v>
+        <v>-9.5926360009204389E-6</v>
       </c>
       <c r="H19">
-        <v>4.4393048925213049E-5</v>
+        <v>3.5676189873261462E-4</v>
       </c>
       <c r="I19">
-        <v>-1.2530241957560461E-4</v>
+        <v>5.6902944001849785E-5</v>
       </c>
       <c r="J19">
-        <v>2.2074305865028154E-4</v>
+        <v>4.0082971452603519E-4</v>
       </c>
       <c r="K19">
-        <v>5.5604009335982404E-5</v>
+        <v>2.4255833903196258E-4</v>
       </c>
       <c r="L19">
-        <v>2.5658339404524035E-4</v>
+        <v>1.7847483114818985E-4</v>
       </c>
       <c r="M19">
-        <v>5.1059293718817671E-4</v>
+        <v>3.7725084422883873E-4</v>
       </c>
       <c r="N19">
-        <v>5.7813511922817987E-4</v>
+        <v>3.0245107304069374E-4</v>
       </c>
       <c r="O19">
-        <v>4.811464463765682E-4</v>
+        <v>-1.4841064432457267E-4</v>
       </c>
       <c r="P19">
-        <v>4.8786060506086958E-4</v>
+        <v>-2.0658737129131653E-4</v>
       </c>
       <c r="Q19">
-        <v>-7.2425620442973676E-4</v>
+        <v>3.0109542111242957E-4</v>
       </c>
       <c r="R19">
-        <v>-3.7907013253733887E-4</v>
+        <v>2.3332758907138713E-4</v>
       </c>
       <c r="S19">
-        <v>8.152753097305799E-4</v>
+        <v>1.2483683570379677E-3</v>
       </c>
       <c r="T19">
-        <v>4.9797153633169495E-3</v>
+        <v>2.8909668466432564E-3</v>
       </c>
       <c r="U19">
-        <v>6.1396227502930056E-4</v>
+        <v>2.0135672055145715E-3</v>
       </c>
       <c r="V19">
-        <v>1.9810284272930552E-4</v>
+        <v>2.1280406399256865E-4</v>
       </c>
       <c r="W19">
-        <v>-1.8447870122822346E-4</v>
+        <v>-3.1412239510812678E-4</v>
       </c>
       <c r="X19">
-        <v>-2.4145573694213059E-4</v>
+        <v>-1.2656278945907731E-4</v>
       </c>
       <c r="Y19">
-        <v>8.0057584316888057E-5</v>
+        <v>6.1825727696772359E-5</v>
       </c>
       <c r="Z19">
-        <v>-2.6731577784837058E-4</v>
+        <v>6.9160869954369361E-5</v>
       </c>
       <c r="AA19">
-        <v>7.9096730570043443E-6</v>
+        <v>4.7610974969589451E-5</v>
       </c>
       <c r="AB19">
-        <v>2.7116128091147975E-5</v>
+        <v>7.3684689751557161E-5</v>
       </c>
       <c r="AC19">
-        <v>4.5098671527915232E-5</v>
+        <v>-1.333637379017402E-4</v>
       </c>
       <c r="AD19">
-        <v>3.9161793982513213E-6</v>
+        <v>-3.0856963767368921E-4</v>
       </c>
       <c r="AE19">
-        <v>-9.7520024108732409E-3</v>
+        <v>-8.7064736070815163E-3</v>
       </c>
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A20" s="4" t="s">
+      <c r="A20" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="4">
-        <v>0.138613214277678</v>
+      <c r="B20">
+        <v>0.69637983266555192</v>
       </c>
       <c r="C20">
-        <v>2.3257402569426891E-4</v>
+        <v>6.7481258606760797E-4</v>
       </c>
       <c r="D20">
-        <v>-2.9933107869743519E-6</v>
+        <v>-1.4569497607665009E-6</v>
       </c>
       <c r="E20">
-        <v>-1.1482362773312244E-3</v>
+        <v>-2.9596719659817005E-3</v>
       </c>
       <c r="F20">
-        <v>-7.9171013475877808E-4</v>
+        <v>3.2629992669071795E-3</v>
       </c>
       <c r="G20">
-        <v>-8.0763066515607794E-4</v>
+        <v>-9.347311100260304E-3</v>
       </c>
       <c r="H20">
-        <v>-1.1885843689452662E-3</v>
+        <v>-1.0010428841263685E-2</v>
       </c>
       <c r="I20">
-        <v>-4.0315965918530892E-5</v>
+        <v>3.4933142166057168E-3</v>
       </c>
       <c r="J20">
-        <v>3.2994248329018538E-5</v>
+        <v>-3.1950436091474632E-3</v>
       </c>
       <c r="K20">
-        <v>5.5119593287239477E-4</v>
+        <v>-7.2647788215747244E-3</v>
       </c>
       <c r="L20">
-        <v>-1.6059617628885747E-4</v>
+        <v>-3.649038641633684E-3</v>
       </c>
       <c r="M20">
-        <v>7.3705097809739772E-4</v>
+        <v>-2.9094610916571284E-3</v>
       </c>
       <c r="N20">
-        <v>5.5518875917112687E-4</v>
+        <v>-4.2623579171752191E-3</v>
       </c>
       <c r="O20">
-        <v>-5.0795982176589762E-4</v>
+        <v>-1.0375994015841185E-2</v>
       </c>
       <c r="P20">
-        <v>2.1220970524371673E-3</v>
+        <v>-7.998476587633821E-3</v>
       </c>
       <c r="Q20">
-        <v>-2.9147874716058033E-4</v>
+        <v>8.82665705467163E-3</v>
       </c>
       <c r="R20">
-        <v>-2.5543451940962122E-3</v>
+        <v>4.0235680416472949E-3</v>
       </c>
       <c r="S20">
-        <v>-5.0083306979949518E-6</v>
+        <v>7.9949883265242883E-3</v>
       </c>
       <c r="T20">
-        <v>6.1396227502930056E-4</v>
+        <v>2.0135672055145715E-3</v>
       </c>
       <c r="U20">
-        <v>6.2611610896891795E-2</v>
+        <v>3.4231343797052176</v>
       </c>
       <c r="V20">
-        <v>-8.4543211326497392E-5</v>
+        <v>-5.7065136194633936E-4</v>
       </c>
       <c r="W20">
-        <v>-1.2299409285449533E-4</v>
+        <v>-9.5619191450737606E-3</v>
       </c>
       <c r="X20">
-        <v>-1.1906319902616792E-4</v>
+        <v>-6.3245886603848778E-3</v>
       </c>
       <c r="Y20">
-        <v>4.5266018432429337E-4</v>
+        <v>-9.7551093127856703E-3</v>
       </c>
       <c r="Z20">
-        <v>3.8195269640143442E-4</v>
+        <v>-5.8251029763756179E-3</v>
       </c>
       <c r="AA20">
-        <v>5.0330488759703189E-4</v>
+        <v>-5.0273970842322768E-3</v>
       </c>
       <c r="AB20">
-        <v>-3.9745613158252062E-4</v>
+        <v>6.3095874666153851E-2</v>
       </c>
       <c r="AC20">
-        <v>-6.5513384018372339E-4</v>
+        <v>8.2458579527455056E-2</v>
       </c>
       <c r="AD20">
-        <v>3.5986587515630906E-3</v>
+        <v>-8.782333296422945E-3</v>
       </c>
       <c r="AE20">
-        <v>-8.2991507920076202E-2</v>
+        <v>-5.6162355854335502</v>
       </c>
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A21" s="4" t="s">
+      <c r="A21" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="4">
-        <v>7.6400911560965096E-2</v>
+      <c r="B21">
+        <v>-0.35436230584910272</v>
       </c>
       <c r="C21">
-        <v>1.036745703606724E-3</v>
+        <v>5.4872781593778841E-4</v>
       </c>
       <c r="D21">
-        <v>-1.417677093281909E-5</v>
+        <v>-7.0509937480622278E-6</v>
       </c>
       <c r="E21">
-        <v>1.1254545305906362E-3</v>
+        <v>1.2881052067806157E-3</v>
       </c>
       <c r="F21">
-        <v>1.7154813598231292E-3</v>
+        <v>1.8284194929131326E-3</v>
       </c>
       <c r="G21">
-        <v>1.8108383199628032E-3</v>
+        <v>2.8534725468392086E-3</v>
       </c>
       <c r="H21">
-        <v>1.7954571935368513E-3</v>
+        <v>3.0473936062167788E-3</v>
       </c>
       <c r="I21">
-        <v>-2.3002156782194079E-4</v>
+        <v>-3.6181095557555679E-4</v>
       </c>
       <c r="J21">
-        <v>-3.1131398564071446E-5</v>
+        <v>4.4284971095989549E-5</v>
       </c>
       <c r="K21">
-        <v>-1.0509328676614957E-4</v>
+        <v>-5.9380501088227011E-4</v>
       </c>
       <c r="L21">
-        <v>3.7888829995916251E-4</v>
+        <v>-3.1392029688528944E-4</v>
       </c>
       <c r="M21">
-        <v>2.5820894272164316E-4</v>
+        <v>-6.1070456127521044E-4</v>
       </c>
       <c r="N21">
-        <v>2.4249225575666625E-4</v>
+        <v>-7.1168020374343111E-4</v>
       </c>
       <c r="O21">
-        <v>6.9032131691097189E-4</v>
+        <v>6.2335694107264845E-4</v>
       </c>
       <c r="P21">
-        <v>4.3644292906844982E-5</v>
+        <v>-5.9864412779825436E-4</v>
       </c>
       <c r="Q21">
-        <v>-1.4736186988996832E-3</v>
+        <v>-6.9298365517534745E-4</v>
       </c>
       <c r="R21">
-        <v>-1.8369318955659765E-4</v>
+        <v>1.3423975894431648E-3</v>
       </c>
       <c r="S21">
-        <v>1.9592037078065437E-4</v>
+        <v>6.1913401883952578E-5</v>
       </c>
       <c r="T21">
-        <v>1.9810284272930552E-4</v>
+        <v>2.1280406399256865E-4</v>
       </c>
       <c r="U21">
-        <v>-8.4543211326497392E-5</v>
+        <v>-5.7065136194633936E-4</v>
       </c>
       <c r="V21">
-        <v>2.5186470893142965E-2</v>
+        <v>4.7047047387407601E-2</v>
       </c>
       <c r="W21">
-        <v>8.6605452987036698E-4</v>
+        <v>1.3382703100489396E-3</v>
       </c>
       <c r="X21">
-        <v>6.4511188072241326E-5</v>
+        <v>1.9969843380792177E-5</v>
       </c>
       <c r="Y21">
-        <v>-2.1972528175086799E-4</v>
+        <v>8.1693866547207297E-4</v>
       </c>
       <c r="Z21">
-        <v>9.1546500222922404E-5</v>
+        <v>3.631621331590465E-4</v>
       </c>
       <c r="AA21">
-        <v>6.6245223789805196E-5</v>
+        <v>4.5075525691440875E-4</v>
       </c>
       <c r="AB21">
-        <v>2.3522284162458171E-5</v>
+        <v>-4.7756520244131122E-5</v>
       </c>
       <c r="AC21">
-        <v>-3.6485347385505074E-7</v>
+        <v>-2.0169701332905989E-4</v>
       </c>
       <c r="AD21">
-        <v>4.2352086338522978E-5</v>
+        <v>-8.3207123552580891E-5</v>
       </c>
       <c r="AE21">
-        <v>-2.0888084053528877E-2</v>
+        <v>-1.1559934617145107E-2</v>
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A22" s="4" t="s">
+      <c r="A22" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="4">
-        <v>-0.10837932836804987</v>
+      <c r="B22">
+        <v>-4.5493998582054371E-2</v>
       </c>
       <c r="C22">
-        <v>8.256034511573869E-5</v>
+        <v>1.3867767885126017E-4</v>
       </c>
       <c r="D22">
-        <v>-9.7725192968876098E-7</v>
+        <v>-2.2688969186693666E-6</v>
       </c>
       <c r="E22">
-        <v>-3.3471972248961439E-5</v>
+        <v>5.6124109139208593E-4</v>
       </c>
       <c r="F22">
-        <v>4.3733593379901355E-4</v>
+        <v>6.4064025476095999E-4</v>
       </c>
       <c r="G22">
-        <v>7.7486338378691662E-4</v>
+        <v>1.7134888506063516E-3</v>
       </c>
       <c r="H22">
-        <v>8.621738419492082E-4</v>
+        <v>2.0052115667627927E-3</v>
       </c>
       <c r="I22">
-        <v>-5.3974580672169834E-5</v>
+        <v>-2.767875043506819E-4</v>
       </c>
       <c r="J22">
-        <v>-1.514370799753645E-4</v>
+        <v>-1.1080150184194208E-4</v>
       </c>
       <c r="K22">
-        <v>-1.7030843422933747E-4</v>
+        <v>-1.7200455675944748E-4</v>
       </c>
       <c r="L22">
-        <v>4.0183811021562987E-4</v>
+        <v>6.3305338590252669E-5</v>
       </c>
       <c r="M22">
-        <v>4.4745943156195706E-4</v>
+        <v>-1.5116710570581976E-4</v>
       </c>
       <c r="N22">
-        <v>4.9592163070215529E-4</v>
+        <v>-6.0703632047888478E-5</v>
       </c>
       <c r="O22">
-        <v>1.4831380963284302E-4</v>
+        <v>4.7680745231862341E-4</v>
       </c>
       <c r="P22">
-        <v>2.7818894293340899E-4</v>
+        <v>5.812671467913188E-4</v>
       </c>
       <c r="Q22">
-        <v>1.6550412430280532E-4</v>
+        <v>3.7250565870342815E-4</v>
       </c>
       <c r="R22">
-        <v>-6.4661622260776255E-6</v>
+        <v>4.2163652572025463E-4</v>
       </c>
       <c r="S22">
-        <v>-1.3280603289883791E-4</v>
+        <v>-3.6821600525828208E-4</v>
       </c>
       <c r="T22">
-        <v>-1.8447870122822346E-4</v>
+        <v>-3.1412239510812678E-4</v>
       </c>
       <c r="U22">
-        <v>-1.2299409285449533E-4</v>
+        <v>-9.5619191450737606E-3</v>
       </c>
       <c r="V22">
-        <v>8.6605452987036698E-4</v>
+        <v>1.3382703100489396E-3</v>
       </c>
       <c r="W22">
-        <v>1.3926431850952248E-3</v>
+        <v>2.2041120805777453E-3</v>
       </c>
       <c r="X22">
-        <v>4.5726485996641208E-5</v>
+        <v>1.1632564856991036E-4</v>
       </c>
       <c r="Y22">
-        <v>1.2236270062001225E-4</v>
+        <v>2.3687198443829265E-4</v>
       </c>
       <c r="Z22">
-        <v>9.0385805348541825E-5</v>
+        <v>3.4509632723331188E-4</v>
       </c>
       <c r="AA22">
-        <v>6.3410483441622473E-5</v>
+        <v>3.1547674107313545E-4</v>
       </c>
       <c r="AB22">
-        <v>5.4576414940648319E-6</v>
+        <v>-2.0618813307545799E-4</v>
       </c>
       <c r="AC22">
-        <v>-8.1539065810655041E-5</v>
+        <v>3.6880647758329762E-5</v>
       </c>
       <c r="AD22">
-        <v>5.568759610072283E-6</v>
+        <v>-3.5070026313477196E-4</v>
       </c>
       <c r="AE22">
-        <v>-2.9693769645715174E-3</v>
+        <v>1.2265932677672115E-2</v>
       </c>
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A23" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23" s="4">
-        <v>-9.3015094325197584E-2</v>
+      <c r="A23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23">
+        <v>-6.848468770174311E-2</v>
       </c>
       <c r="C23">
-        <v>4.255967225028686E-7</v>
+        <v>2.5913086894540846E-5</v>
       </c>
       <c r="D23">
-        <v>-9.8252358527322638E-9</v>
+        <v>-7.9257668560221402E-7</v>
       </c>
       <c r="E23">
-        <v>2.2856607472792245E-4</v>
+        <v>-5.6944476809105203E-4</v>
       </c>
       <c r="F23">
-        <v>2.2090543634875268E-4</v>
+        <v>-4.6659838500573642E-4</v>
       </c>
       <c r="G23">
-        <v>1.4899534601413875E-4</v>
+        <v>5.7599084600067161E-4</v>
       </c>
       <c r="H23">
-        <v>1.3861162955907996E-4</v>
+        <v>6.9347205352700454E-4</v>
       </c>
       <c r="I23">
-        <v>1.596535067560154E-5</v>
+        <v>-7.7850032275234428E-5</v>
       </c>
       <c r="J23">
-        <v>-1.51395986420455E-5</v>
+        <v>-2.9735276442375153E-4</v>
       </c>
       <c r="K23">
-        <v>-3.8045096765947257E-4</v>
+        <v>1.6603513771593775E-4</v>
       </c>
       <c r="L23">
-        <v>-3.7671397780852066E-4</v>
+        <v>7.2134580263658044E-5</v>
       </c>
       <c r="M23">
-        <v>-4.6427709508903119E-4</v>
+        <v>-3.8423601706332605E-4</v>
       </c>
       <c r="N23">
-        <v>-3.9430563060456614E-4</v>
+        <v>-7.0866272852798673E-5</v>
       </c>
       <c r="O23">
-        <v>7.6876093061210106E-5</v>
+        <v>-6.0251583119956499E-5</v>
       </c>
       <c r="P23">
-        <v>-9.6934724572757524E-5</v>
+        <v>2.2828525415892866E-4</v>
       </c>
       <c r="Q23">
-        <v>-2.661655520219098E-4</v>
+        <v>8.0731490063672487E-5</v>
       </c>
       <c r="R23">
-        <v>1.7546977267600099E-4</v>
+        <v>-1.1991082457825809E-4</v>
       </c>
       <c r="S23">
-        <v>-1.0403971901812124E-4</v>
+        <v>-4.6164450322705355E-4</v>
       </c>
       <c r="T23">
-        <v>-2.4145573694213059E-4</v>
+        <v>-1.2656278945907731E-4</v>
       </c>
       <c r="U23">
-        <v>-1.1906319902616792E-4</v>
+        <v>-6.3245886603848778E-3</v>
       </c>
       <c r="V23">
-        <v>6.4511188072241326E-5</v>
+        <v>1.9969843380792177E-5</v>
       </c>
       <c r="W23">
-        <v>4.5726485996641208E-5</v>
+        <v>1.1632564856991036E-4</v>
       </c>
       <c r="X23">
-        <v>2.3963036145122109E-3</v>
+        <v>3.9041223112306163E-3</v>
       </c>
       <c r="Y23">
-        <v>1.1394132423619282E-3</v>
+        <v>2.1033204377843336E-3</v>
       </c>
       <c r="Z23">
-        <v>1.14180093045091E-3</v>
+        <v>1.7861941311982702E-3</v>
       </c>
       <c r="AA23">
-        <v>1.128617649464017E-3</v>
+        <v>1.8520561989303131E-3</v>
       </c>
       <c r="AB23">
-        <v>-1.2986655483020808E-5</v>
+        <v>-1.5171793384304166E-4</v>
       </c>
       <c r="AC23">
-        <v>-4.7846737407848965E-6</v>
+        <v>1.9407337709496857E-4</v>
       </c>
       <c r="AD23">
-        <v>4.7319190284916661E-5</v>
+        <v>-4.4012523390427651E-4</v>
       </c>
       <c r="AE23">
-        <v>-4.4250594001484303E-4</v>
+        <v>9.6168033885531377E-3</v>
       </c>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A24" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24" s="4">
-        <v>-8.8056629631783623E-2</v>
+      <c r="A24" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24">
+        <v>-2.6999425750324418E-2</v>
       </c>
       <c r="C24">
-        <v>-3.4369943042798063E-5</v>
+        <v>9.3965165858727467E-5</v>
       </c>
       <c r="D24">
-        <v>4.5168458805109964E-7</v>
+        <v>-1.4457021524091158E-6</v>
       </c>
       <c r="E24">
-        <v>3.1057699376862123E-4</v>
+        <v>8.8462643243483719E-4</v>
       </c>
       <c r="F24">
-        <v>2.9942339633353343E-4</v>
+        <v>1.1539576645116312E-3</v>
       </c>
       <c r="G24">
-        <v>3.6094664196645993E-4</v>
+        <v>2.0178087705291104E-3</v>
       </c>
       <c r="H24">
-        <v>2.8059981020544682E-4</v>
+        <v>2.275508788050011E-3</v>
       </c>
       <c r="I24">
-        <v>1.0238385191772319E-4</v>
+        <v>-2.9617804134391724E-4</v>
       </c>
       <c r="J24">
-        <v>-7.9660085159065244E-5</v>
+        <v>3.1027127734345765E-5</v>
       </c>
       <c r="K24">
-        <v>-2.4582271198870403E-4</v>
+        <v>-4.778326837388408E-4</v>
       </c>
       <c r="L24">
-        <v>-3.4137581956191192E-4</v>
+        <v>-4.3427722434931371E-4</v>
       </c>
       <c r="M24">
-        <v>-1.9277684255405948E-4</v>
+        <v>-6.121932368545191E-4</v>
       </c>
       <c r="N24">
-        <v>-1.7100302444384395E-4</v>
+        <v>-6.9105148763527746E-4</v>
       </c>
       <c r="O24">
-        <v>1.0344903868390441E-4</v>
+        <v>2.975705552297446E-4</v>
       </c>
       <c r="P24">
-        <v>4.9287291610111998E-4</v>
+        <v>5.1378747704251739E-5</v>
       </c>
       <c r="Q24">
-        <v>-1.5986730426279362E-4</v>
+        <v>-6.399401024035755E-5</v>
       </c>
       <c r="R24">
-        <v>-2.2846398251503505E-4</v>
+        <v>4.3593541650084958E-4</v>
       </c>
       <c r="S24">
-        <v>-5.4826601102152367E-5</v>
+        <v>-2.4991452807371318E-4</v>
       </c>
       <c r="T24">
-        <v>8.0057584316888057E-5</v>
+        <v>6.1825727696772359E-5</v>
       </c>
       <c r="U24">
-        <v>4.5266018432429337E-4</v>
+        <v>-9.7551093127856703E-3</v>
       </c>
       <c r="V24">
-        <v>-2.1972528175086799E-4</v>
+        <v>8.1693866547207297E-4</v>
       </c>
       <c r="W24">
-        <v>1.2236270062001225E-4</v>
+        <v>2.3687198443829265E-4</v>
       </c>
       <c r="X24">
-        <v>1.1394132423619282E-3</v>
+        <v>2.1033204377843336E-3</v>
       </c>
       <c r="Y24">
-        <v>3.3146367685923141E-3</v>
+        <v>5.2768462651535553E-3</v>
       </c>
       <c r="Z24">
-        <v>1.126972949342196E-3</v>
+        <v>1.7453396151478637E-3</v>
       </c>
       <c r="AA24">
-        <v>1.1399084708895184E-3</v>
+        <v>1.8162323490049325E-3</v>
       </c>
       <c r="AB24">
-        <v>-1.1819314082355626E-5</v>
+        <v>-2.1742628443621075E-4</v>
       </c>
       <c r="AC24">
-        <v>-1.0156273015465917E-4</v>
+        <v>-1.5960144898752266E-4</v>
       </c>
       <c r="AD24">
-        <v>4.5358370753200562E-5</v>
+        <v>-5.6658596963453291E-4</v>
       </c>
       <c r="AE24">
-        <v>-1.1450566768274675E-3</v>
+        <v>1.2483790353955623E-2</v>
       </c>
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A25" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B25" s="4">
-        <v>1.306812135078203E-2</v>
+      <c r="A25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25">
+        <v>6.611732298753259E-2</v>
       </c>
       <c r="C25">
-        <v>5.7247109565838894E-6</v>
+        <v>-1.6917361960915034E-4</v>
       </c>
       <c r="D25">
-        <v>1.5333999195543346E-8</v>
+        <v>2.4065892310144482E-6</v>
       </c>
       <c r="E25">
-        <v>1.7767527515970575E-4</v>
+        <v>-3.6064803144921593E-5</v>
       </c>
       <c r="F25">
-        <v>1.9853308174726752E-4</v>
+        <v>-2.7223485210811898E-4</v>
       </c>
       <c r="G25">
-        <v>2.2530322637951653E-4</v>
+        <v>3.111905074119673E-4</v>
       </c>
       <c r="H25">
-        <v>2.605508110060199E-4</v>
+        <v>3.1228006393693979E-4</v>
       </c>
       <c r="I25">
-        <v>3.4609419491087924E-5</v>
+        <v>-2.7750551696720379E-4</v>
       </c>
       <c r="J25">
-        <v>5.1172868672602211E-5</v>
+        <v>-6.2188839705147776E-5</v>
       </c>
       <c r="K25">
-        <v>-1.284220570935005E-4</v>
+        <v>-3.8246733922961407E-4</v>
       </c>
       <c r="L25">
-        <v>-1.2230621992551528E-4</v>
+        <v>-3.3983709615911795E-4</v>
       </c>
       <c r="M25">
-        <v>-1.3906646043800389E-4</v>
+        <v>-5.6821633514136938E-4</v>
       </c>
       <c r="N25">
-        <v>-1.4266392760561245E-4</v>
+        <v>-3.3076199473364154E-4</v>
       </c>
       <c r="O25">
-        <v>8.3212268812885487E-5</v>
+        <v>2.5410061215240445E-4</v>
       </c>
       <c r="P25">
-        <v>2.1397395422366526E-4</v>
+        <v>3.4452728579310258E-4</v>
       </c>
       <c r="Q25">
-        <v>-8.3156147322452931E-5</v>
+        <v>-2.9044001037349838E-4</v>
       </c>
       <c r="R25">
-        <v>-8.2324881837983325E-5</v>
+        <v>4.08985385420748E-5</v>
       </c>
       <c r="S25">
-        <v>-2.3388965619314977E-5</v>
+        <v>-3.1266888160362202E-4</v>
       </c>
       <c r="T25">
-        <v>-2.6731577784837058E-4</v>
+        <v>6.9160869954369361E-5</v>
       </c>
       <c r="U25">
-        <v>3.8195269640143442E-4</v>
+        <v>-5.8251029763756179E-3</v>
       </c>
       <c r="V25">
-        <v>9.1546500222922404E-5</v>
+        <v>3.631621331590465E-4</v>
       </c>
       <c r="W25">
-        <v>9.0385805348541825E-5</v>
+        <v>3.4509632723331188E-4</v>
       </c>
       <c r="X25">
-        <v>1.14180093045091E-3</v>
+        <v>1.7861941311982702E-3</v>
       </c>
       <c r="Y25">
-        <v>1.126972949342196E-3</v>
+        <v>1.7453396151478637E-3</v>
       </c>
       <c r="Z25">
-        <v>2.4034957567781387E-3</v>
+        <v>2.7388737757088116E-3</v>
       </c>
       <c r="AA25">
-        <v>1.136619478606092E-3</v>
+        <v>1.6972782942771014E-3</v>
       </c>
       <c r="AB25">
-        <v>-2.4725432462594121E-5</v>
+        <v>-1.7270325029185616E-4</v>
       </c>
       <c r="AC25">
-        <v>2.7851526926298562E-5</v>
+        <v>1.5641171722602024E-4</v>
       </c>
       <c r="AD25">
-        <v>9.8701359849394127E-5</v>
+        <v>-2.6754133944927722E-4</v>
       </c>
       <c r="AE25">
-        <v>-1.6252374383883749E-3</v>
+        <v>1.2542017481454802E-2</v>
       </c>
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A26" s="4" t="s">
+      <c r="A26" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="4">
-        <v>-4.3127899685774435E-2</v>
+      <c r="B26">
+        <v>-8.6944866979451113E-2</v>
       </c>
       <c r="C26">
-        <v>-1.5838513064547559E-5</v>
+        <v>-3.875855575427925E-5</v>
       </c>
       <c r="D26">
-        <v>2.6570736051742815E-7</v>
+        <v>3.0475044868048156E-7</v>
       </c>
       <c r="E26">
-        <v>2.8429778853909923E-4</v>
+        <v>1.555712424833489E-4</v>
       </c>
       <c r="F26">
-        <v>2.7598110523056212E-4</v>
+        <v>-1.6058912491110668E-4</v>
       </c>
       <c r="G26">
-        <v>3.9546046006957644E-4</v>
+        <v>5.2490679053886951E-4</v>
       </c>
       <c r="H26">
-        <v>4.0835041409025886E-4</v>
+        <v>7.0290194679995498E-4</v>
       </c>
       <c r="I26">
-        <v>3.9438556723504873E-5</v>
+        <v>-2.165427260908937E-4</v>
       </c>
       <c r="J26">
-        <v>-1.7265724705360424E-5</v>
+        <v>-1.6239261766208763E-4</v>
       </c>
       <c r="K26">
-        <v>4.6902342506572204E-4</v>
+        <v>2.5723409530692409E-5</v>
       </c>
       <c r="L26">
-        <v>-1.0161682224577289E-4</v>
+        <v>-1.5114739733154692E-4</v>
       </c>
       <c r="M26">
-        <v>-4.9608189989342431E-5</v>
+        <v>-3.9098676380741604E-4</v>
       </c>
       <c r="N26">
-        <v>3.8489258457458618E-5</v>
+        <v>-1.8219403422939373E-4</v>
       </c>
       <c r="O26">
-        <v>4.962905437433277E-5</v>
+        <v>2.6284742542824436E-4</v>
       </c>
       <c r="P26">
-        <v>-4.8228911015247774E-6</v>
+        <v>1.6895230994670891E-4</v>
       </c>
       <c r="Q26">
-        <v>-5.6907486115411382E-5</v>
+        <v>-2.877600456760495E-4</v>
       </c>
       <c r="R26">
-        <v>1.7121583925899119E-4</v>
+        <v>2.5207197076730983E-5</v>
       </c>
       <c r="S26">
-        <v>4.2485836602178115E-5</v>
+        <v>-3.3986133414734814E-4</v>
       </c>
       <c r="T26">
-        <v>7.9096730570043443E-6</v>
+        <v>4.7610974969589451E-5</v>
       </c>
       <c r="U26">
-        <v>5.0330488759703189E-4</v>
+        <v>-5.0273970842322768E-3</v>
       </c>
       <c r="V26">
-        <v>6.6245223789805196E-5</v>
+        <v>4.5075525691440875E-4</v>
       </c>
       <c r="W26">
-        <v>6.3410483441622473E-5</v>
+        <v>3.1547674107313545E-4</v>
       </c>
       <c r="X26">
-        <v>1.128617649464017E-3</v>
+        <v>1.8520561989303131E-3</v>
       </c>
       <c r="Y26">
-        <v>1.1399084708895184E-3</v>
+        <v>1.8162323490049325E-3</v>
       </c>
       <c r="Z26">
-        <v>1.136619478606092E-3</v>
+        <v>1.6972782942771014E-3</v>
       </c>
       <c r="AA26">
-        <v>1.6759501026546804E-3</v>
+        <v>2.7756221090144495E-3</v>
       </c>
       <c r="AB26">
-        <v>-1.3352418916546307E-5</v>
+        <v>-1.5561456830912235E-4</v>
       </c>
       <c r="AC26">
-        <v>2.4982273494333625E-5</v>
+        <v>2.6432586247279223E-4</v>
       </c>
       <c r="AD26">
-        <v>5.3013328795380545E-5</v>
+        <v>-2.9390360070430903E-4</v>
       </c>
       <c r="AE26">
-        <v>-1.8101207599157086E-3</v>
+        <v>8.87242350477754E-3</v>
       </c>
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A27" s="4" t="s">
+      <c r="A27" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="4">
-        <v>1.8471480415839833E-2</v>
+      <c r="B27">
+        <v>-1.2445048803401693E-2</v>
       </c>
       <c r="C27">
-        <v>5.9137605493958998E-6</v>
+        <v>2.7676159033733147E-5</v>
       </c>
       <c r="D27">
-        <v>-1.1857098752095007E-7</v>
+        <v>-2.0298817239389688E-7</v>
       </c>
       <c r="E27">
-        <v>-1.5808479232049642E-5</v>
+        <v>-4.1240557598391076E-5</v>
       </c>
       <c r="F27">
-        <v>-1.4929545295904917E-5</v>
+        <v>7.8199851678291627E-5</v>
       </c>
       <c r="G27">
-        <v>-2.6689480399168821E-6</v>
+        <v>-1.9824853210931477E-4</v>
       </c>
       <c r="H27">
-        <v>6.4342486495588409E-6</v>
+        <v>-2.275053647680643E-4</v>
       </c>
       <c r="I27">
-        <v>-2.7214548413133252E-6</v>
+        <v>7.9762339600379759E-5</v>
       </c>
       <c r="J27">
-        <v>-2.7829571149668148E-6</v>
+        <v>-2.1941907255594692E-5</v>
       </c>
       <c r="K27">
-        <v>-2.8285873803390448E-5</v>
+        <v>-1.2153932766847259E-4</v>
       </c>
       <c r="L27">
-        <v>-1.3468760293948025E-5</v>
+        <v>-6.3188053292702329E-5</v>
       </c>
       <c r="M27">
-        <v>-3.8728019827620447E-5</v>
+        <v>-3.1311804414090039E-5</v>
       </c>
       <c r="N27">
-        <v>-3.7190050698999972E-5</v>
+        <v>-7.879956687860401E-5</v>
       </c>
       <c r="O27">
-        <v>4.1569522667938513E-5</v>
+        <v>-2.2960068732225786E-4</v>
       </c>
       <c r="P27">
-        <v>-3.8323392250187401E-5</v>
+        <v>-1.8890471060084807E-4</v>
       </c>
       <c r="Q27">
-        <v>-3.8230551777755741E-5</v>
+        <v>1.6316875023124995E-4</v>
       </c>
       <c r="R27">
-        <v>3.086857548289209E-5</v>
+        <v>7.5724639217917417E-5</v>
       </c>
       <c r="S27">
-        <v>1.5451025931629641E-5</v>
+        <v>1.9454093844275947E-4</v>
       </c>
       <c r="T27">
-        <v>2.7116128091147975E-5</v>
+        <v>7.3684689751557161E-5</v>
       </c>
       <c r="U27">
-        <v>-3.9745613158252062E-4</v>
+        <v>6.3095874666153851E-2</v>
       </c>
       <c r="V27">
-        <v>2.3522284162458171E-5</v>
+        <v>-4.7756520244131122E-5</v>
       </c>
       <c r="W27">
-        <v>5.4576414940648319E-6</v>
+        <v>-2.0618813307545799E-4</v>
       </c>
       <c r="X27">
-        <v>-1.2986655483020808E-5</v>
+        <v>-1.5171793384304166E-4</v>
       </c>
       <c r="Y27">
-        <v>-1.1819314082355626E-5</v>
+        <v>-2.1742628443621075E-4</v>
       </c>
       <c r="Z27">
-        <v>-2.4725432462594121E-5</v>
+        <v>-1.7270325029185616E-4</v>
       </c>
       <c r="AA27">
-        <v>-1.3352418916546307E-5</v>
+        <v>-1.5561456830912235E-4</v>
       </c>
       <c r="AB27">
-        <v>2.6983569595569837E-5</v>
+        <v>1.2013423749410966E-3</v>
       </c>
       <c r="AC27">
-        <v>-1.0462852695158201E-4</v>
+        <v>1.3158745148023898E-3</v>
       </c>
       <c r="AD27">
-        <v>-1.555754373125941E-4</v>
+        <v>-4.1345549131951553E-4</v>
       </c>
       <c r="AE27">
-        <v>1.0539250620569688E-4</v>
+        <v>-0.10441329849340564</v>
       </c>
     </row>
     <row r="28" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A28" s="4" t="s">
+      <c r="A28" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="4">
-        <v>3.7713558541715229E-2</v>
+      <c r="B28">
+        <v>1.4552076719212425E-2</v>
       </c>
       <c r="C28">
-        <v>5.159375546955015E-5</v>
+        <v>-2.8837001124054889E-4</v>
       </c>
       <c r="D28">
-        <v>-8.1506749543800876E-7</v>
+        <v>3.7089664899785427E-6</v>
       </c>
       <c r="E28">
-        <v>2.3912491505732447E-4</v>
+        <v>-3.3106782533749848E-4</v>
       </c>
       <c r="F28">
-        <v>-3.279483099759891E-5</v>
+        <v>-3.8058554416651037E-4</v>
       </c>
       <c r="G28">
-        <v>1.3158211822331036E-5</v>
+        <v>-1.1234744616190403E-4</v>
       </c>
       <c r="H28">
-        <v>5.1524792219336413E-5</v>
+        <v>-1.7836881509195371E-4</v>
       </c>
       <c r="I28">
-        <v>-2.5578364481533339E-5</v>
+        <v>-4.8693203654902339E-5</v>
       </c>
       <c r="J28">
-        <v>-3.9288890784926135E-5</v>
+        <v>-2.9354741869922976E-4</v>
       </c>
       <c r="K28">
-        <v>1.2965498805307535E-3</v>
+        <v>6.4573110388512628E-4</v>
       </c>
       <c r="L28">
-        <v>-6.8579148196939999E-5</v>
+        <v>1.084405486169622E-3</v>
       </c>
       <c r="M28">
-        <v>-5.9849585982117703E-5</v>
+        <v>7.1781241283169067E-4</v>
       </c>
       <c r="N28">
-        <v>-1.1601445814387462E-4</v>
+        <v>9.289849170115716E-4</v>
       </c>
       <c r="O28">
-        <v>-5.2681368138991151E-4</v>
+        <v>-2.0857481001030124E-5</v>
       </c>
       <c r="P28">
-        <v>1.7784775603164904E-4</v>
+        <v>5.5571748364532448E-4</v>
       </c>
       <c r="Q28">
-        <v>4.545165394622421E-4</v>
+        <v>3.222092623969895E-4</v>
       </c>
       <c r="R28">
-        <v>-3.1174316931970438E-4</v>
+        <v>-4.4206742426121902E-4</v>
       </c>
       <c r="S28">
-        <v>1.1634006715949784E-4</v>
+        <v>-1.3531950853782064E-4</v>
       </c>
       <c r="T28">
-        <v>4.5098671527915232E-5</v>
+        <v>-1.333637379017402E-4</v>
       </c>
       <c r="U28">
-        <v>-6.5513384018372339E-4</v>
+        <v>8.2458579527455056E-2</v>
       </c>
       <c r="V28">
-        <v>-3.6485347385505074E-7</v>
+        <v>-2.0169701332905989E-4</v>
       </c>
       <c r="W28">
-        <v>-8.1539065810655041E-5</v>
+        <v>3.6880647758329762E-5</v>
       </c>
       <c r="X28">
-        <v>-4.7846737407848965E-6</v>
+        <v>1.9407337709496857E-4</v>
       </c>
       <c r="Y28">
-        <v>-1.0156273015465917E-4</v>
+        <v>-1.5960144898752266E-4</v>
       </c>
       <c r="Z28">
-        <v>2.7851526926298562E-5</v>
+        <v>1.5641171722602024E-4</v>
       </c>
       <c r="AA28">
-        <v>2.4982273494333625E-5</v>
+        <v>2.6432586247279223E-4</v>
       </c>
       <c r="AB28">
-        <v>-1.0462852695158201E-4</v>
+        <v>1.3158745148023898E-3</v>
       </c>
       <c r="AC28">
-        <v>3.2376679397965007E-3</v>
+        <v>1.0209771673958271E-2</v>
       </c>
       <c r="AD28">
-        <v>8.3715384164173752E-4</v>
+        <v>1.3874063229439059E-3</v>
       </c>
       <c r="AE28">
-        <v>1.5120088370187438E-3</v>
+        <v>-0.12726289467461438</v>
       </c>
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A29" s="4" t="s">
+      <c r="A29" t="s">
         <v>14</v>
       </c>
-      <c r="B29" s="4">
-        <v>1.0680613465932139E-2</v>
+      <c r="B29">
+        <v>4.3120410636546876E-2</v>
       </c>
       <c r="C29">
-        <v>2.5710270849494711E-5</v>
+        <v>-8.8906726277164852E-5</v>
       </c>
       <c r="D29">
-        <v>-4.0582316391967095E-7</v>
+        <v>1.0264545465087224E-6</v>
       </c>
       <c r="E29">
-        <v>3.1818351229789257E-4</v>
+        <v>1.9770032406867682E-4</v>
       </c>
       <c r="F29">
-        <v>2.3388041275380824E-4</v>
+        <v>3.3909788902428654E-4</v>
       </c>
       <c r="G29">
-        <v>1.7514425447485776E-4</v>
+        <v>-3.9797461241870326E-4</v>
       </c>
       <c r="H29">
-        <v>1.6785572366683236E-4</v>
+        <v>-3.5256610842830015E-4</v>
       </c>
       <c r="I29">
-        <v>-5.9407444466610905E-5</v>
+        <v>-2.8823954779161811E-5</v>
       </c>
       <c r="J29">
-        <v>-3.1125863325718868E-5</v>
+        <v>-2.8384302803011391E-4</v>
       </c>
       <c r="K29">
-        <v>1.7246407844620504E-4</v>
+        <v>-7.1332150796014036E-5</v>
       </c>
       <c r="L29">
-        <v>-2.1924498427777772E-5</v>
+        <v>8.4224755973066195E-5</v>
       </c>
       <c r="M29">
-        <v>1.2623628609969434E-4</v>
+        <v>1.2550409944924509E-4</v>
       </c>
       <c r="N29">
-        <v>1.4057615879197946E-4</v>
+        <v>-1.0482830196222558E-5</v>
       </c>
       <c r="O29">
-        <v>-1.1693663405852828E-4</v>
+        <v>-3.2755124765183712E-4</v>
       </c>
       <c r="P29">
-        <v>1.2564404886540901E-4</v>
+        <v>-3.36103046794762E-4</v>
       </c>
       <c r="Q29">
-        <v>-8.3217073198970336E-6</v>
+        <v>1.978664787983278E-4</v>
       </c>
       <c r="R29">
-        <v>-2.4049389922529464E-4</v>
+        <v>7.7905155236683771E-5</v>
       </c>
       <c r="S29">
-        <v>1.2973870902276401E-6</v>
+        <v>4.2491279157220584E-5</v>
       </c>
       <c r="T29">
-        <v>3.9161793982513213E-6</v>
+        <v>-3.0856963767368921E-4</v>
       </c>
       <c r="U29">
-        <v>3.5986587515630906E-3</v>
+        <v>-8.782333296422945E-3</v>
       </c>
       <c r="V29">
-        <v>4.2352086338522978E-5</v>
+        <v>-8.3207123552580891E-5</v>
       </c>
       <c r="W29">
-        <v>5.568759610072283E-6</v>
+        <v>-3.5070026313477196E-4</v>
       </c>
       <c r="X29">
-        <v>4.7319190284916661E-5</v>
+        <v>-4.4012523390427651E-4</v>
       </c>
       <c r="Y29">
-        <v>4.5358370753200562E-5</v>
+        <v>-5.6658596963453291E-4</v>
       </c>
       <c r="Z29">
-        <v>9.8701359849394127E-5</v>
+        <v>-2.6754133944927722E-4</v>
       </c>
       <c r="AA29">
-        <v>5.3013328795380545E-5</v>
+        <v>-2.9390360070430903E-4</v>
       </c>
       <c r="AB29">
-        <v>-1.555754373125941E-4</v>
+        <v>-4.1345549131951553E-4</v>
       </c>
       <c r="AC29">
-        <v>8.3715384164173752E-4</v>
+        <v>1.3874063229439059E-3</v>
       </c>
       <c r="AD29">
-        <v>3.3083323387292302E-3</v>
+        <v>1.1826716374992389E-2</v>
       </c>
       <c r="AE29">
-        <v>-3.3889965547701691E-3</v>
+        <v>2.0273257185484346E-2</v>
       </c>
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.45">
-      <c r="A30" s="4" t="s">
+      <c r="A30" t="s">
         <v>15</v>
       </c>
-      <c r="B30" s="4">
-        <v>-2.9088969591501219</v>
+      <c r="B30">
+        <v>-4.3252847747838725</v>
       </c>
       <c r="C30">
-        <v>-1.3815079267640334E-2</v>
+        <v>-2.4829431322037993E-2</v>
       </c>
       <c r="D30">
-        <v>1.9533488433813129E-4</v>
+        <v>3.2634569391603403E-4</v>
       </c>
       <c r="E30">
-        <v>-1.2059508707464417E-2</v>
+        <v>-1.2387257461297358E-2</v>
       </c>
       <c r="F30">
-        <v>-8.55532189017464E-3</v>
+        <v>-2.2905120743896279E-2</v>
       </c>
       <c r="G30">
-        <v>-7.707975565897307E-3</v>
+        <v>9.8791132255200004E-4</v>
       </c>
       <c r="H30">
-        <v>-7.6562263933973307E-3</v>
+        <v>-7.1839709934884421E-4</v>
       </c>
       <c r="I30">
-        <v>4.6719183804137653E-3</v>
+        <v>-9.458810079688261E-4</v>
       </c>
       <c r="J30">
-        <v>-2.4581550854899849E-3</v>
+        <v>4.0779576794641205E-3</v>
       </c>
       <c r="K30">
-        <v>-8.2742245904287581E-2</v>
+        <v>-6.9344512243916911E-2</v>
       </c>
       <c r="L30">
-        <v>-8.2753910604096759E-2</v>
+        <v>-7.592401252361336E-2</v>
       </c>
       <c r="M30">
-        <v>-8.4244609024092143E-2</v>
+        <v>-7.4408123300112816E-2</v>
       </c>
       <c r="N30">
-        <v>-8.3793811011936059E-2</v>
+        <v>-6.980181834357313E-2</v>
       </c>
       <c r="O30">
-        <v>-6.2254617512547822E-4</v>
+        <v>2.5008630614879075E-2</v>
       </c>
       <c r="P30">
-        <v>8.6616340823723252E-4</v>
+        <v>1.6504489093138681E-2</v>
       </c>
       <c r="Q30">
-        <v>-8.4558287762910578E-4</v>
+        <v>-2.1883668073604076E-2</v>
       </c>
       <c r="R30">
-        <v>3.7602632527530353E-3</v>
+        <v>-1.0053438042088594E-2</v>
       </c>
       <c r="S30">
-        <v>-4.2793830195181314E-3</v>
+        <v>-1.6196901215115495E-2</v>
       </c>
       <c r="T30">
-        <v>-9.7520024108732409E-3</v>
+        <v>-8.7064736070815163E-3</v>
       </c>
       <c r="U30">
-        <v>-8.2991507920076202E-2</v>
+        <v>-5.6162355854335502</v>
       </c>
       <c r="V30">
-        <v>-2.0888084053528877E-2</v>
+        <v>-1.1559934617145107E-2</v>
       </c>
       <c r="W30">
-        <v>-2.9693769645715174E-3</v>
+        <v>1.2265932677672115E-2</v>
       </c>
       <c r="X30">
-        <v>-4.4250594001484303E-4</v>
+        <v>9.6168033885531377E-3</v>
       </c>
       <c r="Y30">
-        <v>-1.1450566768274675E-3</v>
+        <v>1.2483790353955623E-2</v>
       </c>
       <c r="Z30">
-        <v>-1.6252374383883749E-3</v>
+        <v>1.2542017481454802E-2</v>
       </c>
       <c r="AA30">
-        <v>-1.8101207599157086E-3</v>
+        <v>8.87242350477754E-3</v>
       </c>
       <c r="AB30">
-        <v>1.0539250620569688E-4</v>
+        <v>-0.10441329849340564</v>
       </c>
       <c r="AC30">
-        <v>1.5120088370187438E-3</v>
+        <v>-0.12726289467461438</v>
       </c>
       <c r="AD30">
-        <v>-3.3889965547701691E-3</v>
+        <v>2.0273257185484346E-2</v>
       </c>
       <c r="AE30">
-        <v>0.44023385203122389</v>
+        <v>9.7461169630096833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new edits from daria
</commit_message>
<xml_diff>
--- a/input/reg_fertility.xlsx
+++ b/input/reg_fertility.xlsx
@@ -8,8 +8,8 @@
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId2"/>
     <sheet name="Gof" sheetId="2" r:id="rId4"/>
-    <sheet name="F1a" sheetId="3" r:id="rId5"/>
-    <sheet name="F1b" sheetId="4" r:id="rId6"/>
+    <sheet name="UK_F1a" sheetId="3" r:id="rId5"/>
+    <sheet name="UK_F1b" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>

</xml_diff>